<commit_message>
add circulatory system artery and vein data
</commit_message>
<xml_diff>
--- a/ai/data/raw/Project_CirculatorySystem_EDatas.xlsx
+++ b/ai/data/raw/Project_CirculatorySystem_EDatas.xlsx
@@ -1,17 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/ee662cdd26a9269a/Masaüstü/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="11_04540A0CEF3E18847B4A8305486F9BDB5CAD2C2A" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet state="visible" name="Sayfa1" sheetId="1" r:id="rId5"/>
+    <sheet name="Sayfa1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="271" uniqueCount="136">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="953" uniqueCount="451">
   <si>
     <t>id</t>
   </si>
@@ -419,24 +428,971 @@
   </si>
   <si>
     <t>["Bu kas tabakası kasılarak kanın kalpten damarlara pompalanmasını sağlar."]</t>
+  </si>
+  <si>
+    <t>arteries</t>
+  </si>
+  <si>
+    <t>Atardamarlar</t>
+  </si>
+  <si>
+    <t>Vessels</t>
+  </si>
+  <si>
+    <t>artery; arter; vessel; blood circulation; damar</t>
+  </si>
+  <si>
+    <t>Atardamarlar, kanı kalpten dokulara ve organlara taşıyan kan damarlarıdır.</t>
+  </si>
+  <si>
+    <t>["Atardamarlar kalbin ventrikülleri ile bağlantılı damarlardır ve kanı kalpten uzaklaştırarak vücudun farklı bölgelerine taşırlar.", "Sağ ventrikülden akciğerlere kirli kan taşıyan akciğer atardamarı dışında diğer tüm atardamarlar oksijen bakımından zengin temiz kan taşır.", "Sol ventrikülden çıkan temiz kan sistol sırasında aort damarına pompalanır ve buradan vücuttaki diğer atardamarlara dağıtılır.", "Atardamarların çapları perifer bölgelere doğru gidildikçe küçülür ve bu küçük damarlara arteriyol adı verilir.", "Atardamarlarda kan basıncı yüksek olduğu için damar duvarları toplardamarlara göre daha kalın ve dayanıklıdır."]</t>
+  </si>
+  <si>
+    <t>Ders kitabı s.138</t>
+  </si>
+  <si>
+    <t>upper_extremity_arteries</t>
+  </si>
+  <si>
+    <t>Üst ekstremite arterleri</t>
+  </si>
+  <si>
+    <t>Upper_Extremity</t>
+  </si>
+  <si>
+    <t>artery; arter; upper extremity; arm; kol; damar; subclavian; axillary; brachial; radial; ulnar</t>
+  </si>
+  <si>
+    <t>Üst ekstremite arterleri, omuzdan ele kadar üst ekstremiteyi besleyen atardamarlardır.</t>
+  </si>
+  <si>
+    <t>["Sağ ve sol köprücük altı arterleri kola doğru ilerledikçe çapları giderek küçülür ve geçtikleri bölgeye göre farklı isimler alırlar.","Üst ekstremitede arterler sırasıyla a. subclavia, a. axillaris, a. brachialis, a. radialis ve a. ulnaris olarak devam eder.","Bu damarlar omuz, kol, ön kol ve elin kanlanmasını sağlar."]</t>
+  </si>
+  <si>
+    <t>subclavian_artery</t>
+  </si>
+  <si>
+    <t>A. subclavia</t>
+  </si>
+  <si>
+    <t>artery; subclavian artery; a. subclavia; upper extremity; arter; köprücük altı atardamarı;atardamar</t>
+  </si>
+  <si>
+    <t>A. subclavia, üst ekstremiteye kan taşıyan ana arterlerden biridir.</t>
+  </si>
+  <si>
+    <t>["Sağ ve sol a. subclavia, üst ekstremiteye uzanan arteriyel dolaşımın başlangıç bölümünü oluşturur.","Bu damar kola doğru ilerledikçe bulunduğu bölgeye göre isim değiştirir.","Koltuk altı bölgesine ulaştığında a. axillaris adını alır."]</t>
+  </si>
+  <si>
+    <t>axillary_artery</t>
+  </si>
+  <si>
+    <t>A. axillaris</t>
+  </si>
+  <si>
+    <t>artery; arter; axillary artery; a. axillaris; koltuk altı atardamarı; upper extremity;atardamar</t>
+  </si>
+  <si>
+    <t>A. axillaris, a. subclavia'nın koltuk altı bölgesindeki devamıdır.</t>
+  </si>
+  <si>
+    <t>["A. subclavia, koltuk altı bölgesine geldiğinde a. axillaris adını alır.","A. axillaris göğüs ve omuz bölgesine dallar verir.","Bu damar kol bölgesine doğru devam ederek a. brachialis adını alır."]</t>
+  </si>
+  <si>
+    <t>brachial_artery</t>
+  </si>
+  <si>
+    <t>A. brachialis</t>
+  </si>
+  <si>
+    <t>artery; arter; brachial artery; a. brachialis; kol atardamarı; blood pressure;atardamar</t>
+  </si>
+  <si>
+    <t>A. brachialis, a. axillaris'in kol bölgesindeki devamıdır.</t>
+  </si>
+  <si>
+    <t>["A. axillaris kol bölgesine geçince a. brachialis adını alır.","A. brachialis kol kaslarının beslenmesini sağlar.","Tansiyon ölçümü klinikte bu damar üzerinden yapılır.","Dirsek ön bölgesinde a. radialis ve a. ulnaris olmak üzere iki dala ayrılır."]</t>
+  </si>
+  <si>
+    <t>radial_artery</t>
+  </si>
+  <si>
+    <t>A. radialis</t>
+  </si>
+  <si>
+    <t>artery; arter; radial artery; a. radialis; radius; nabız; pulse; upper extremity;atardamar</t>
+  </si>
+  <si>
+    <t>A. radialis, a. brachialis'in dirsek ön bölgesinde ayrılan dallarından biridir.</t>
+  </si>
+  <si>
+    <t>["A. brachialis dirsek ön bölgesinde a. radialis ve a. ulnaris olarak iki dala ayrılır.","A. radialis ön kolun ve elin bir bölümünün kanlanmasına katkı sağlar.","A. radialis nabız almada daha sık tercih edilen damarlardan biridir."]</t>
+  </si>
+  <si>
+    <t>ulnar_artery</t>
+  </si>
+  <si>
+    <t>A. ulnaris</t>
+  </si>
+  <si>
+    <t>artery; arter; ulnar artery; a. ulnaris; ulna; upper extremity;atardamar</t>
+  </si>
+  <si>
+    <t>A. ulnaris, a. brachialis'in dirsek ön bölgesinde ayrılan dallarından biridir.</t>
+  </si>
+  <si>
+    <t>["A. brachialis dirsek ön bölgesinde iki ana dala ayrılır ve bunlardan biri a. ulnaris'tir.","A. ulnaris ön kolun ve elin bir bölümünün kanlanmasına katkı sağlar.","A. ulnaris, a. radialis ile birlikte el bileği ve elin beslenmesinde görev alır."]</t>
+  </si>
+  <si>
+    <t>abdominal_aorta</t>
+  </si>
+  <si>
+    <t>Karın aortu</t>
+  </si>
+  <si>
+    <t>Abdomen</t>
+  </si>
+  <si>
+    <t>artery; abdominal aorta; aorta abdominalis; circulation; abdomen;atardamar</t>
+  </si>
+  <si>
+    <t>Karın aortu, aortun diyaframdan sonra karın boşluğunda devam eden bölümüdür.</t>
+  </si>
+  <si>
+    <t>["Karın aortu diyaframdan başlayarak bel omurları boyunca aşağı doğru uzanır.","Bu damar karın bölgesindeki birçok organa kan taşıyan arterlerin çıktığı ana damardır.","Truncus coeliacus, a. mesenterica superior ve a. mesenterica inferior gibi önemli arterler karın aortundan ayrılır.","Karın aortu yaklaşık dördüncü bel omuru hizasında ikiye ayrılarak sağ ve sol a. iliaca communis arterlerini oluşturur."]</t>
+  </si>
+  <si>
+    <t>truncus_coeliacus</t>
+  </si>
+  <si>
+    <t>Truncus coeliacus</t>
+  </si>
+  <si>
+    <t>artery; truncus coeliacus; celiac trunk; abdominal aorta;atardamar</t>
+  </si>
+  <si>
+    <t>Truncus coeliacus, karın aortundan ayrılan ve üç ana dala ayrılan önemli bir arterdir.</t>
+  </si>
+  <si>
+    <t>["Truncus coeliacus karın aortundan ayrılır.","Bu damar üç ana dala ayrılarak karın bölgesindeki bazı organlara kan taşır.","Dalları mide, karaciğer ve dalak gibi organların beslenmesine katkı sağlar."]</t>
+  </si>
+  <si>
+    <t>gastrica_sinistra</t>
+  </si>
+  <si>
+    <t>A. gastrica sinistra</t>
+  </si>
+  <si>
+    <t>artery; gastrica sinistra; left gastric artery; stomach;atardamar</t>
+  </si>
+  <si>
+    <t>A. gastrica sinistra, mideyi besleyen arterlerden biridir</t>
+  </si>
+  <si>
+    <t>["Bu damar karın aortundan çıkan truncus coeliacusun dallarından biridir.","Midenin üst kısmına kan taşır.","Mide duvarının beslenmesine katkı sağlar."]</t>
+  </si>
+  <si>
+    <t>hepatica_communis</t>
+  </si>
+  <si>
+    <t>A. hepatica communis</t>
+  </si>
+  <si>
+    <t>artery; hepatica communis; common hepatic artery; liver;atardamar</t>
+  </si>
+  <si>
+    <t>A. hepatica communis, karaciğeri besleyen önemli arterlerden biridir.</t>
+  </si>
+  <si>
+    <t>["Bu damar truncus coeliacusun ana dallarından biridir.","Karaciğere kan taşır.","Karaciğer dokusunun beslenmesinde görev alır."]</t>
+  </si>
+  <si>
+    <t>lienalis</t>
+  </si>
+  <si>
+    <t>A. lienalis</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> artery; lienalis; splenic artery; spleen; pancreas;atardamar</t>
+  </si>
+  <si>
+    <t>A. lienalis, dalak ve pankreası besleyen arterlerden biridir.</t>
+  </si>
+  <si>
+    <t>["Bu damar truncus coeliacusun dallarından biridir.","Dalak dokusuna kan taşır.","Pankreasın bir bölümünün beslenmesine katkı sağlar."]</t>
+  </si>
+  <si>
+    <t>mesenterica_superior</t>
+  </si>
+  <si>
+    <t>A. mesenterica superior</t>
+  </si>
+  <si>
+    <t>artery; mesenterica superior; superior mesenteric artery; intestine;atardamar</t>
+  </si>
+  <si>
+    <t>A. mesenterica superior, ince bağırsak ve kalın bağırsağın bir bölümünü besleyen arterdir.</t>
+  </si>
+  <si>
+    <t>["Bu damar karın aortundan ayrılır.","İnce bağırsağa kan taşır.","Kalın bağırsağın ilk yarısının beslenmesine katkı sağlar."]</t>
+  </si>
+  <si>
+    <t>mesenterica_inferior</t>
+  </si>
+  <si>
+    <t>A. mesenterica inferior</t>
+  </si>
+  <si>
+    <t>artery; mesenterica inferior; inferior mesenteric artery; intestine;atardamar</t>
+  </si>
+  <si>
+    <t>A. mesenterica inferior, kalın bağırsağın ikinci yarısını besleyen arterdir.</t>
+  </si>
+  <si>
+    <t>["Bu damar karın aortundan ayrılır.","Kalın bağırsağın alt bölümlerine kan taşır.","Sindirim sisteminin alt kısmının beslenmesinde görev alır."]</t>
+  </si>
+  <si>
+    <t>renalis</t>
+  </si>
+  <si>
+    <t>A. renalis</t>
+  </si>
+  <si>
+    <t>artery; renalis; renal artery; kidney;atardamar</t>
+  </si>
+  <si>
+    <t>A. renalis, böbreklere kan taşıyan büyük arterlerden biridir.</t>
+  </si>
+  <si>
+    <t>["Bu damar karın aortundan ayrılır.","Böbreklere oksijen bakımından zengin kan taşır.","Böbrek dokusunun beslenmesinde önemli rol oynar."]</t>
+  </si>
+  <si>
+    <t>gonadal_artery</t>
+  </si>
+  <si>
+    <t>A. testicularis / A. ovarica</t>
+  </si>
+  <si>
+    <t>artery; testicular artery; ovarian artery; gonadal artery;atardamar</t>
+  </si>
+  <si>
+    <t>A. testicularis ve A. ovarica, üreme organlarını besleyen arterlerdir.</t>
+  </si>
+  <si>
+    <t>["Bu damarlar karın aortundan ayrılır.","Erkeklerde testislerin kanlanmasını sağlar.","Kadınlarda yumurtalıkların beslenmesinde görev alır."]</t>
+  </si>
+  <si>
+    <t>lumbales</t>
+  </si>
+  <si>
+    <t>A. lumbales</t>
+  </si>
+  <si>
+    <t>artery; lumbales; lumbar artery; spine;atardamar</t>
+  </si>
+  <si>
+    <t>A. lumbales, bel bölgesindeki yapıları besleyen arterlerdir.</t>
+  </si>
+  <si>
+    <t>["Bu damarlar karın aortundan ayrılır.","Omurilik çevresindeki kas ve dokulara kan taşırlar.","Bel bölgesinin kanlanmasına katkı sağlarlar."]</t>
+  </si>
+  <si>
+    <t>sacralis_media</t>
+  </si>
+  <si>
+    <t>A. sacralis media</t>
+  </si>
+  <si>
+    <t>artery; sacralis media; sacral artery; sacrum;atardamar</t>
+  </si>
+  <si>
+    <t>A. sacralis media, sakrum bölgesini besleyen arterdir</t>
+  </si>
+  <si>
+    <t>["Bu damar karın aortunun alt kısmından ayrılır.","Sakrum bölgesine kan taşır.","Pelvis bölgesindeki bazı yapıların beslenmesine katkı sağlar."]</t>
+  </si>
+  <si>
+    <t>phrenica_inferior</t>
+  </si>
+  <si>
+    <t>A. phrenica inferior</t>
+  </si>
+  <si>
+    <t>artery; phrenica inferior; inferior phrenic artery; diaphragm;atardamar</t>
+  </si>
+  <si>
+    <t>A. phrenica inferior, diyaframın alt kısmını besleyen arterlerden biridir.</t>
+  </si>
+  <si>
+    <t>["Bu damar karın aortundan ayrılır.","Diyaframın alt yüzüne kan taşır.","Diyafram kasının beslenmesinde görev alır."]</t>
+  </si>
+  <si>
+    <t>iliaca_communis</t>
+  </si>
+  <si>
+    <t>A. iliaca communis</t>
+  </si>
+  <si>
+    <t>Lower_Extremity</t>
+  </si>
+  <si>
+    <t>artery; iliaca communis; common iliac artery; pelvis; atardamar</t>
+  </si>
+  <si>
+    <t>A. iliaca communis, karın aortunun ikiye ayrılmasıyla oluşan büyük arterlerden biridir.</t>
+  </si>
+  <si>
+    <t>["Karın aortu yaklaşık dördüncü bel omuru hizasında ikiye ayrılarak sağ ve sol a. iliaca communis arterlerini oluşturur.","Bu arter pelvis bölgesine doğru ilerler.","Pelvis içinde a. iliaca interna ve a. iliaca externa olmak üzere iki ana dala ayrılır."]</t>
+  </si>
+  <si>
+    <t>Ders kitabı s.139</t>
+  </si>
+  <si>
+    <t>iliaca_interna</t>
+  </si>
+  <si>
+    <t>A. iliaca internus</t>
+  </si>
+  <si>
+    <t>artery; iliaca interna; internal iliac artery; pelvis; atardamar</t>
+  </si>
+  <si>
+    <t>A. iliaca interna, pelvis boşluğundaki organları besleyen arterdir.</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> ["Bu damar a. iliaca communisin dallarından biridir.","Pelvis boşluğu içinde ilerler.","Mesane, rektum ve pelvis kasları gibi yapılara dallar vererek bu bölgelerin beslenmesini sağlar."]</t>
+  </si>
+  <si>
+    <t>iliaca_externa</t>
+  </si>
+  <si>
+    <t>A. iliaca externus</t>
+  </si>
+  <si>
+    <t>artery; iliaca externa; external iliac artery; leg; atardamar</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> A. iliaca externa, alt ekstremiteye kan taşıyan önemli arterlerden biridir.</t>
+  </si>
+  <si>
+    <t>["Bu damar a. iliaca communisin iki ana dalından biridir.","Pelvis bölgesinden çıkarak bacaklara doğru ilerler.","Alt ekstremitenin kanlanmasını sağlayan arteriyel dolaşımın devamını oluşturur."]</t>
+  </si>
+  <si>
+    <t>femoralis</t>
+  </si>
+  <si>
+    <t>A. femoralis</t>
+  </si>
+  <si>
+    <t>artery; femoralis; femoral artery; thigh; atardamar</t>
+  </si>
+  <si>
+    <t>A. femoralis, uyluk bölgesini besleyen büyük bir arterdir.</t>
+  </si>
+  <si>
+    <t>["A. iliaca externa uyluk bölgesine ulaştığında a. femoralis adını alır.","Bu arter uyluk kaslarına dallar vererek bölgenin kanlanmasını sağlar.","Uyluk boyunca aşağı doğru ilerleyerek diz bölgesine ulaşır."]</t>
+  </si>
+  <si>
+    <t>poplitea</t>
+  </si>
+  <si>
+    <t>A. poplitea</t>
+  </si>
+  <si>
+    <t>artery; poplitea; popliteal artery; knee; atardamar</t>
+  </si>
+  <si>
+    <t>A. poplitea, diz arkasında bulunan ve diz bölgesini besleyen arterdir.</t>
+  </si>
+  <si>
+    <t>["A. femoralis diz bölgesine ulaştığında a. poplitea adını alır.","Bu arter dizin arka kısmında yer alır.","Diz çevresindeki yapıların beslenmesini sağlar."]</t>
+  </si>
+  <si>
+    <t>tibialis_anterior</t>
+  </si>
+  <si>
+    <t>A. tibialis anterior</t>
+  </si>
+  <si>
+    <t>artery; tibialis anterior; anterior tibial artery; leg; atardamar</t>
+  </si>
+  <si>
+    <t>A. tibialis anterior, bacağın ön kısmını besleyen arterdir.</t>
+  </si>
+  <si>
+    <t>["A. poplitea baldır bölgesinde iki ana dala ayrılır.","Bu dallardan biri a. tibialis anteriordur.","Bacağın ön kısmındaki kasların ve dokuların beslenmesini sağlar.","Ayak sırtında a. dorsalis pedis olarak devam eder."]</t>
+  </si>
+  <si>
+    <t>tibialis_posterior</t>
+  </si>
+  <si>
+    <t>A. tibialis posterior</t>
+  </si>
+  <si>
+    <t>artery; tibialis posterior; posterior tibial artery; leg; atardamar</t>
+  </si>
+  <si>
+    <t>A. tibialis posterior, bacağın arka bölümünü besleyen arterdir.</t>
+  </si>
+  <si>
+    <t>["A. poplitea baldır bölgesinde a. tibialis anterior ve a. tibialis posterior olarak ikiye ayrılır.","A. tibialis posterior bacağın arka bölümündeki kasları besler.","Alt bacak ve ayak bölgesinin kanlanmasına katkı sağlar."]</t>
+  </si>
+  <si>
+    <t>dorsalis_pedis</t>
+  </si>
+  <si>
+    <t>A. dorsalis pedis</t>
+  </si>
+  <si>
+    <t>artery; dorsalis pedis; foot artery; pulse; atardamar</t>
+  </si>
+  <si>
+    <t>A. dorsalis pedis, ayağın üst kısmında bulunan arterdir.</t>
+  </si>
+  <si>
+    <t>["A. tibialis anterior ayak sırtına ulaştığında a. dorsalis pedis adını alır.","Ayağın üst kısmındaki dokuların beslenmesini sağlar.","Birinci metatarsal aralıkta bu arter üzerinden nabız alınabilir."]</t>
+  </si>
+  <si>
+    <t>temporalis</t>
+  </si>
+  <si>
+    <t>A. temporalis</t>
+  </si>
+  <si>
+    <t>Head_Face</t>
+  </si>
+  <si>
+    <t>artery; temporalis; temporal artery; nabız; atardamar</t>
+  </si>
+  <si>
+    <t>A. temporalis, baş bölgesinde nabız alınabilen arterlerden biridir.</t>
+  </si>
+  <si>
+    <t>["Bu arter şakak bölgesinde bulunur.","Baş bölgesinde nabız değerlendirilirken bu damardan yararlanılabilir."]</t>
+  </si>
+  <si>
+    <t>Ders kitabı s.143</t>
+  </si>
+  <si>
+    <t>carotis_communis</t>
+  </si>
+  <si>
+    <t>A. carotis communis</t>
+  </si>
+  <si>
+    <t>Neck</t>
+  </si>
+  <si>
+    <t>artery; carotis communis; carotid artery; nabız; atardamar</t>
+  </si>
+  <si>
+    <t>A. carotis communis, boyun bölgesinde nabız alınabilen önemli arterlerden biridir.</t>
+  </si>
+  <si>
+    <t>["Bu arter boyunda yer alır.","Fiziksel muayenede karotis arterden nabız alınabilir.","Karotis arterden nabız alınırken dikkat edilmelidir."]</t>
+  </si>
+  <si>
+    <t>axillaris_pulse</t>
+  </si>
+  <si>
+    <t>artery; axillaris; axillary artery; nabız; atardamar</t>
+  </si>
+  <si>
+    <t>A. axillaris, üst ekstremitede nabız alınabilen arterlerden biridir.</t>
+  </si>
+  <si>
+    <t>["Bu arter koltuk altı bölgesinde bulunur.","Üst ekstremite arterlerinden biri olarak nabız değerlendirmesinde kullanılabilir."]</t>
+  </si>
+  <si>
+    <t>brachialis_pulse</t>
+  </si>
+  <si>
+    <t>artery; brachialis; brachial artery; nabız; atardamar</t>
+  </si>
+  <si>
+    <t>A. brachialis, üst ekstremitede nabız alınabilen arterlerden biridir.</t>
+  </si>
+  <si>
+    <t>["Bu arter kol bölgesinde bulunur.","Fiziksel muayenede üst ekstremite arterlerinden biri olarak nabız değerlendirilmesinde kullanılabilir."]</t>
+  </si>
+  <si>
+    <t>ulnaris_pulse</t>
+  </si>
+  <si>
+    <t>artery; ulnaris; ulnar artery; nabız; atardamar</t>
+  </si>
+  <si>
+    <t>A. ulnaris, ön kol bölgesinde bulunan arterlerden biridir.</t>
+  </si>
+  <si>
+    <t>["Bu arter ön kol bölgesinde yer alır.","Üst ekstremitede nabız alınabilen arterlerden biridir."]</t>
+  </si>
+  <si>
+    <t>radialis_pulse</t>
+  </si>
+  <si>
+    <t>artery; radialis; radial artery; nabız; atardamar</t>
+  </si>
+  <si>
+    <t>A. radialis, el bileğinde nabız alınmasında yaygın olarak kullanılan arterdir.</t>
+  </si>
+  <si>
+    <t>["Bu arter el bileği bölgesinde bulunur.","Rutin muayenelerde nabız genellikle radial arter üzerinden değerlendirilir."]</t>
+  </si>
+  <si>
+    <t>femoralis_pulse</t>
+  </si>
+  <si>
+    <t>artery; femoralis; femoral artery; nabız; atardamar</t>
+  </si>
+  <si>
+    <t>A. femoralis, alt ekstremitede nabız alınabilen arterlerden biridir.</t>
+  </si>
+  <si>
+    <t>["Bu arter uyluk bölgesinde bulunur.","Alt ekstremite arterlerinden biri olarak nabız değerlendirilmesinde kullanılabilir."]</t>
+  </si>
+  <si>
+    <t>poplitea_pulse</t>
+  </si>
+  <si>
+    <t>artery; poplitea; popliteal artery; nabız; atardamar</t>
+  </si>
+  <si>
+    <t>A. poplitea, diz arkasında bulunan arterdir.</t>
+  </si>
+  <si>
+    <t>["Bu arter dizin arka kısmında yer alır.","Alt ekstremitede nabız değerlendirilirken bu damardan yararlanılabilir."]</t>
+  </si>
+  <si>
+    <t>tibialis_posterior_pulse</t>
+  </si>
+  <si>
+    <t>artery; tibialis posterior; posterior tibial artery; nabız; atardamar</t>
+  </si>
+  <si>
+    <t>A. tibialis posterior, alt bacak bölgesinde nabız alınabilen arterlerden biridir.</t>
+  </si>
+  <si>
+    <t>["Bu arter baldır bölgesinde yer alır.","Alt ekstremitede nabız değerlendirilmesinde kullanılan arterlerden biridir."]</t>
+  </si>
+  <si>
+    <t>dorsalis_pedis_pulse</t>
+  </si>
+  <si>
+    <t>Foot</t>
+  </si>
+  <si>
+    <t>artery; dorsalis pedis; foot artery; nabız; atardamar</t>
+  </si>
+  <si>
+    <t>["Bu arter ayak sırtında bulunur.","Alt ekstremitede nabız değerlendirilirken bu damardan yararlanılabilir."]</t>
+  </si>
+  <si>
+    <t>veins</t>
+  </si>
+  <si>
+    <t>Toplardamarlar</t>
+  </si>
+  <si>
+    <t>vein; vena; ven; circulation; toplardamar</t>
+  </si>
+  <si>
+    <t>Toplardamarlar, kanı dokular ve akciğerlerden kalbe taşıyan damar grubudur.</t>
+  </si>
+  <si>
+    <t>["Temiz kanı akciğerlerden kalbe taşıyan akciğer toplardamarları dışında venler kirli kan taşır.","Venlerde kan basıncı arterlere göre daha düşüktür.","Ven duvarları arterlere göre daha incedir.","Normal istirahat halinde dolaşımdaki kanın büyük bir bölümü venlerde bulunur."]</t>
+  </si>
+  <si>
+    <t>Ders kitabı s.140</t>
+  </si>
+  <si>
+    <t>upper_extremity_veins</t>
+  </si>
+  <si>
+    <t>Üst ekstremite venleri</t>
+  </si>
+  <si>
+    <t>vein; upper extremity veins; arm veins; vena; toplardamar</t>
+  </si>
+  <si>
+    <t>Üst ekstremite venleri, kol bölgesindeki kirli kanı kalbe doğru taşıyan toplardamarlardır.</t>
+  </si>
+  <si>
+    <t>["Üst ekstremite venleri yüzeysel ve derin venler olmak üzere iki grupta incelenir.","Yüzeysel venler deri altında seyreder ve görülebilir.","Önemli yüzeysel venler arasında v. cephalica, v. basilica, v. mediana antebrachii ve v. mediana cubiti bulunur.","Derin venler arterlerle birlikte seyreder.","Önemli derin venler arasında v. radialis, v. ulnaris, v. brachialis ve v. axillaris yer alır.","Üst ekstremiteden gelen venöz kan v. subclavia üzerinden daha büyük venlere taşınır."]</t>
+  </si>
+  <si>
+    <t>brachiocephalica_vein</t>
+  </si>
+  <si>
+    <t>V. brachiocephalica</t>
+  </si>
+  <si>
+    <t>vein; brachiocephalica; brachiocephalic vein; toplardamar</t>
+  </si>
+  <si>
+    <t>V. brachiocephalica, kol ve baş bölgesinden gelen venlerin birleşmesi ile oluşur.</t>
+  </si>
+  <si>
+    <t>["Baş bölgesinden gelen v. jugularis interna ile boynun dış venlerinden v. jugularis externa birleşir.","Koldan gelen v. subclavia ile birleşerek v. brachiocephalica oluşur."]</t>
+  </si>
+  <si>
+    <t>jugularis_interna</t>
+  </si>
+  <si>
+    <t>V. jugularis interna</t>
+  </si>
+  <si>
+    <t>vein; jugularis interna; internal jugular vein; toplardamar</t>
+  </si>
+  <si>
+    <t>V. jugularis interna boyundaki en büyük vendir.</t>
+  </si>
+  <si>
+    <t>["Beyin venleri ile baş bölgesinin derin venlerini birleştirir.","Karotis arter ile komşu olarak boyundan aşağı doğru ilerler.","V. subclavia ile birleşir."]</t>
+  </si>
+  <si>
+    <t>jugularis_externa</t>
+  </si>
+  <si>
+    <t>V. jugularis externa</t>
+  </si>
+  <si>
+    <t>vein; jugularis externa; external jugular vein; toplardamar</t>
+  </si>
+  <si>
+    <t>V. jugularis externa başın dış venlerini ve yüzün yüzeysel venlerini toplar.</t>
+  </si>
+  <si>
+    <t>["Baş ve yüzün yüzeysel venleri ile birleşir.","Boyundan aşağı doğru ilerler.","V. subclavia ile birleşerek sonlanır."]</t>
+  </si>
+  <si>
+    <t>subclavia_vein</t>
+  </si>
+  <si>
+    <t>V. subclavia</t>
+  </si>
+  <si>
+    <t>vein; subclavia; subclavian vein; toplardamar</t>
+  </si>
+  <si>
+    <t>V. subclavia, kol venlerinin birleşmesi ile oluşan vendir.</t>
+  </si>
+  <si>
+    <t>["Kol venleri birleşerek v. axillaris'i oluşturur.","V. axillaris köprücük kemiğinin altında v. subclavia adını alır.","Buradan jugular venlerle birleşerek v. brachiocephalica'yı oluşturur."]</t>
+  </si>
+  <si>
+    <t>axillaris_vein</t>
+  </si>
+  <si>
+    <t>V. axillaris</t>
+  </si>
+  <si>
+    <t>vein; axillaris; axillary vein; toplardamar</t>
+  </si>
+  <si>
+    <t>V. axillaris kol venlerinin birleşmesi ile oluşan vendir.</t>
+  </si>
+  <si>
+    <t>["Kol bölgesindeki venlerin birleşmesi ile oluşur.","Koltuk altı bölgesinde bulunur.","Yukarı doğru ilerleyerek v. subclavia olarak devam eder."]</t>
+  </si>
+  <si>
+    <t>cephalica_vein</t>
+  </si>
+  <si>
+    <t>V. cephalica</t>
+  </si>
+  <si>
+    <t>vein; cephalica; cephalic vein; toplardamar</t>
+  </si>
+  <si>
+    <t>V. cephalica üst ekstremitenin önemli yüzeysel venlerinden biridir.</t>
+  </si>
+  <si>
+    <t>["El sırtının radyal tarafından başlar.","Ön kolun ön tarafına doğru ilerler.","Kolun dış yanından yukarı çıkar.","Proksimalde v. axillarise katılır."]</t>
+  </si>
+  <si>
+    <t>brachialis_vein</t>
+  </si>
+  <si>
+    <t>V. brachialis</t>
+  </si>
+  <si>
+    <t>vein; brachialis; brachial vein; toplardamar</t>
+  </si>
+  <si>
+    <t>V. brachialis kol bölgesinin derin venlerinden biridir.</t>
+  </si>
+  <si>
+    <t>["V. radialis ve v. ulnarisin dirsek önünde birleşmesi ile oluşur.","Yukarı doğru ilerleyerek v. axillarise katılır."]</t>
+  </si>
+  <si>
+    <t>basilica_vein</t>
+  </si>
+  <si>
+    <t>V. basilica</t>
+  </si>
+  <si>
+    <t>vein; basilica; basilic vein; toplardamar</t>
+  </si>
+  <si>
+    <t>V. basilica üst ekstremitenin önemli yüzeysel venlerinden biridir.</t>
+  </si>
+  <si>
+    <t>["El sırtının ulnar tarafından başlar.","Ön kolun iç yüzünden yukarı doğru ilerler.","Dirsek bölgesini geçerek kol bölgesine ulaşır.","Kol bölgesinde derine girerek v. axillaris adını alır."]</t>
+  </si>
+  <si>
+    <t>mediana_cubiti</t>
+  </si>
+  <si>
+    <t>V. mediana cubiti</t>
+  </si>
+  <si>
+    <t>vein; mediana cubiti; median cubital vein; toplardamar</t>
+  </si>
+  <si>
+    <t>V. mediana cubiti dirsek bölgesinde bulunan yüzeysel vendir.</t>
+  </si>
+  <si>
+    <t>["Dirsek ekleminin iç yüzünde bulunur.","V. basilica ile v. cephalicayı birbirine bağlar."]</t>
+  </si>
+  <si>
+    <t>antebrachii_mediana</t>
+  </si>
+  <si>
+    <t>V. antebrachii mediana</t>
+  </si>
+  <si>
+    <t>vein; antebrachii mediana; median antebrachial vein; toplardamar</t>
+  </si>
+  <si>
+    <t>V. antebrachii mediana ön kolun yüzeysel venlerinden biridir.</t>
+  </si>
+  <si>
+    <t>["Elin palmar yüzünden başlayarak yukarı doğru uzanır.","V. mediana cubiti veya v. basilica ile birleşir."]</t>
+  </si>
+  <si>
+    <t>radialis_vein</t>
+  </si>
+  <si>
+    <t>V. radialis</t>
+  </si>
+  <si>
+    <t>vein; radialis; radial vein; toplardamar</t>
+  </si>
+  <si>
+    <t>V. radialis el ve ön kolun radyal bölgesinin venöz kanını toplar.</t>
+  </si>
+  <si>
+    <t>["El ve ön kolun radyal tarafındaki kirli kanı toplar.","V. ulnaris ile birleşerek v. brachialisi oluşturur."]</t>
+  </si>
+  <si>
+    <t>ulnaris_vein</t>
+  </si>
+  <si>
+    <t>V. ulnaris</t>
+  </si>
+  <si>
+    <t>vein; ulnaris; ulnar vein; toplardamar</t>
+  </si>
+  <si>
+    <t>V. ulnaris el ve ön kolun ulnar bölgesinin venöz kanını toplar.</t>
+  </si>
+  <si>
+    <t>["El ve ön kolun ulnar tarafındaki kirli kanı toplar.","V. radialis ile birleşerek v. brachialisi oluşturur."]</t>
+  </si>
+  <si>
+    <t>cava_superior</t>
+  </si>
+  <si>
+    <t>V. cava superior</t>
+  </si>
+  <si>
+    <t>Thorax</t>
+  </si>
+  <si>
+    <t>vein; cava superior; superior vena cava; toplardamar</t>
+  </si>
+  <si>
+    <t>V. cava superior, baş, boyun, göğüs ve üst ekstremite bölgelerinden gelen venöz kanı kalbe taşıyan büyük bir toplardamardır.</t>
+  </si>
+  <si>
+    <t>["V. cava superior iki adet v. brachiocephalicanın birleşmesi ile oluşur.","Baş, boyun, göğüs ve üst ekstremite bölgelerinden gelen kirli kanı toplar.","Topladığı kanı kalbin sağ atriumuna taşır."]</t>
+  </si>
+  <si>
+    <t>lower_extremity_veins</t>
+  </si>
+  <si>
+    <t>Alt ekstremite venleri</t>
+  </si>
+  <si>
+    <t>vein; lower extremity veins; leg veins; vena; toplardamar</t>
+  </si>
+  <si>
+    <t>Alt ekstremite venleri bacak ve ayak bölgesindeki venöz kanı kalbe doğru taşıyan toplardamarlardır.</t>
+  </si>
+  <si>
+    <t>["Alt ekstremite venleri yüzeysel ve derin venler olmak üzere iki grupta incelenir.","Yüzeysel venlerin yapısında kapakçıklar bulunur.","Derin venler genellikle aynı isimdeki arterlerle birlikte seyreder.","Alt ekstremiteden gelen venöz kan daha büyük venler aracılığıyla v. cava inferiora taşınır."]</t>
+  </si>
+  <si>
+    <t>Ders kitabı s.141</t>
+  </si>
+  <si>
+    <t>cava_inferior</t>
+  </si>
+  <si>
+    <t>V. cava inferior</t>
+  </si>
+  <si>
+    <t>vein; cava inferior; inferior vena cava; toplardamar</t>
+  </si>
+  <si>
+    <t>V. cava inferior gövdenin alt bölümünden gelen venöz kanı kalbe taşıyan büyük bir vendir.</t>
+  </si>
+  <si>
+    <t>["Gövdede diyaframın altında kalan bölüm ile alt ekstremite bölgelerinin kanını toplar.","Sağ ve sol v. iliaca communisin birleşmesi ile oluşur.","Topladığı kanı kalbin sağ atriumuna taşır."]</t>
+  </si>
+  <si>
+    <t>iliaca_communis_vein</t>
+  </si>
+  <si>
+    <t>V. iliaca communis</t>
+  </si>
+  <si>
+    <t>Pelvis</t>
+  </si>
+  <si>
+    <t>vein; iliaca communis; common iliac vein; toplardamar</t>
+  </si>
+  <si>
+    <t>V. iliaca communis pelvis ve alt ekstremitenin venöz kanını taşıyan vendir.</t>
+  </si>
+  <si>
+    <t>["V. iliaca interna ve v. iliaca externa venlerinin birleşmesi ile oluşur.","Sağ ve sol v. iliaca communis venleri birleşerek v. cava inferioru oluşturur."]</t>
+  </si>
+  <si>
+    <t>iliaca_externa_vein</t>
+  </si>
+  <si>
+    <t>V. iliaca externa</t>
+  </si>
+  <si>
+    <t>vein; iliaca externa; external iliac vein; toplardamar</t>
+  </si>
+  <si>
+    <t>V. iliaca externa alt ekstremitenin venöz kanını taşıyan önemli venlerden biridir.</t>
+  </si>
+  <si>
+    <t>["Alt ekstremiteden gelen venöz kanı taşır.","Kasık bölgesinden aşağıda v. femoralis adını alır."]</t>
+  </si>
+  <si>
+    <t>femoralis_vein</t>
+  </si>
+  <si>
+    <t>V. femoralis</t>
+  </si>
+  <si>
+    <t>vein; femoralis; femoral vein; toplardamar</t>
+  </si>
+  <si>
+    <t>V. femoralis bacak bölgesinin venöz kanını taşıyan önemli derin vendir.</t>
+  </si>
+  <si>
+    <t>["Bacak bölgesinin kirli kanını taşır.","V. popliteanın devamıdır.","Yukarı doğru ilerleyerek kasık bölgesinde v. iliaca externa adını alır."]</t>
+  </si>
+  <si>
+    <t>poplitea_vein</t>
+  </si>
+  <si>
+    <t>V. poplitea</t>
+  </si>
+  <si>
+    <t>vein; poplitea; popliteal vein; toplardamar</t>
+  </si>
+  <si>
+    <t>V. poplitea diz arkasında bulunan derin vendir.</t>
+  </si>
+  <si>
+    <t>["V. tibialis anterior ve v. tibialis posteriorun birleşmesi ile oluşur.","Diz arkasından yukarı doğru ilerler.","Yukarıda v. femoralis adını alır."]</t>
+  </si>
+  <si>
+    <t>tibialis_anterior_vein</t>
+  </si>
+  <si>
+    <t>V. tibialis anterior</t>
+  </si>
+  <si>
+    <t>vein; tibialis anterior; anterior tibial vein; toplardamar</t>
+  </si>
+  <si>
+    <t>V. tibialis anterior ayak ve bacağın ön bölümünden gelen venöz kanı taşır.</t>
+  </si>
+  <si>
+    <t>["Ayak sırtından başlayarak baldırın önünden yukarı doğru ilerler.","V. tibialis posterior ile birleşerek v. popliteayı oluşturur."]</t>
+  </si>
+  <si>
+    <t>tibialis_posterior_vein</t>
+  </si>
+  <si>
+    <t>V. tibialis posterior</t>
+  </si>
+  <si>
+    <t>vein; tibialis posterior; posterior tibial vein; toplardamar</t>
+  </si>
+  <si>
+    <t>V. tibialis posterior ayak tabanı ve baldır bölgesinin venöz kanını taşır.</t>
+  </si>
+  <si>
+    <t>["Ayak tabanından başlayarak baldırın arka kısmından yukarı doğru ilerler.","V. tibialis anterior ile birleşerek v. popliteayı oluşturur."]</t>
+  </si>
+  <si>
+    <t>saphena_magna</t>
+  </si>
+  <si>
+    <t>V. saphena magna</t>
+  </si>
+  <si>
+    <t>vein; saphena magna; great saphenous vein; toplardamar</t>
+  </si>
+  <si>
+    <t>V. saphena magna vücudun en uzun venidir.</t>
+  </si>
+  <si>
+    <t>["Ayak sırtından başlar.","Bacağın iç yüzünden yukarı doğru ilerler.","Kasık bölgesinde v. femoralis ile birleşir.","Koroner arter bypass ameliyatlarında greft olarak kullanılabilir."]</t>
+  </si>
+  <si>
+    <t>saphena_parva</t>
+  </si>
+  <si>
+    <t>V. saphena parva</t>
+  </si>
+  <si>
+    <t>vein; saphena parva; small saphenous vein; toplardamar</t>
+  </si>
+  <si>
+    <t>V. saphena parva alt ekstremitenin yüzeysel venlerinden biridir.</t>
+  </si>
+  <si>
+    <t>["Ayak sırtının dış tarafından başlar.","Baldırın arka kısmından yukarı doğru ilerler.","Diz arkasında derine ilerleyerek v. popliteaya bağlanır."]</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="3">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
-      <sz val="10.0"/>
+      <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
     </font>
     <font>
+      <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
       <scheme val="minor"/>
@@ -447,43 +1403,44 @@
       <patternFill patternType="none"/>
     </fill>
     <fill>
-      <patternFill patternType="lightGray"/>
+      <patternFill patternType="gray125"/>
     </fill>
   </fills>
   <borders count="1">
-    <border/>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="3">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle xfId="0" name="Normal" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<x18tc:personList xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments"/>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheets">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Sheets">
   <a:themeElements>
     <a:clrScheme name="Sheets">
       <a:dk1>
@@ -673,17 +1630,20 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <dimension ref="A1:N87"/>
+  <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -718,7 +1678,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>11</v>
       </c>
@@ -753,7 +1713,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="3">
+    <row r="3" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>22</v>
       </c>
@@ -785,7 +1745,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="4">
+    <row r="4" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>27</v>
       </c>
@@ -817,7 +1777,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="5">
+    <row r="5" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>31</v>
       </c>
@@ -852,7 +1812,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="6">
+    <row r="6" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>37</v>
       </c>
@@ -887,7 +1847,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="7">
+    <row r="7" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>42</v>
       </c>
@@ -922,7 +1882,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="8">
+    <row r="8" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>47</v>
       </c>
@@ -957,7 +1917,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="9">
+    <row r="9" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>52</v>
       </c>
@@ -992,7 +1952,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="10">
+    <row r="10" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>57</v>
       </c>
@@ -1024,7 +1984,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="11">
+    <row r="11" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>62</v>
       </c>
@@ -1056,7 +2016,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="12">
+    <row r="12" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>66</v>
       </c>
@@ -1091,7 +2051,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="13">
+    <row r="13" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>71</v>
       </c>
@@ -1126,7 +2086,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="14">
+    <row r="14" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>76</v>
       </c>
@@ -1161,7 +2121,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="15">
+    <row r="15" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>82</v>
       </c>
@@ -1196,7 +2156,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="16">
+    <row r="16" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>87</v>
       </c>
@@ -1231,7 +2191,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="17">
+    <row r="17" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
         <v>92</v>
       </c>
@@ -1266,7 +2226,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="18">
+    <row r="18" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
         <v>97</v>
       </c>
@@ -1302,7 +2262,7 @@
       </c>
       <c r="N18" s="2"/>
     </row>
-    <row r="19">
+    <row r="19" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
         <v>102</v>
       </c>
@@ -1337,7 +2297,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="20">
+    <row r="20" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
         <v>106</v>
       </c>
@@ -1372,7 +2332,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="21">
+    <row r="21" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
         <v>110</v>
       </c>
@@ -1407,7 +2367,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="22">
+    <row r="22" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
         <v>115</v>
       </c>
@@ -1442,7 +2402,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="23">
+    <row r="23" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
         <v>121</v>
       </c>
@@ -1477,7 +2437,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="24">
+    <row r="24" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
         <v>126</v>
       </c>
@@ -1512,7 +2472,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="25">
+    <row r="25" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
         <v>131</v>
       </c>
@@ -1547,7 +2507,2177 @@
         <v>120</v>
       </c>
     </row>
+    <row r="26" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C26" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D26" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E26" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="F26" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="G26" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="H26" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="I26" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="J26" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="K26" s="2" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="27" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C27" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D27" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E27" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="F27" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="G27" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="H27" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="I27" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="J27" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="K27" s="2" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="28" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C28" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D28" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="E28" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="F28" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="G28" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="H28" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="I28" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="J28" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="K28" s="2" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="29" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C29" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D29" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="E29" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="F29" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="G29" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="H29" s="2" t="s">
+        <v>156</v>
+      </c>
+      <c r="I29" s="2" t="s">
+        <v>157</v>
+      </c>
+      <c r="J29" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="K29" s="2" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="30" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="2" t="s">
+        <v>159</v>
+      </c>
+      <c r="B30" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C30" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D30" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="E30" s="2" t="s">
+        <v>160</v>
+      </c>
+      <c r="F30" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="G30" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="H30" s="2" t="s">
+        <v>161</v>
+      </c>
+      <c r="I30" s="2" t="s">
+        <v>162</v>
+      </c>
+      <c r="J30" s="2" t="s">
+        <v>163</v>
+      </c>
+      <c r="K30" s="2" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="31" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="B31" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C31" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D31" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="E31" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="F31" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="G31" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="H31" s="2" t="s">
+        <v>166</v>
+      </c>
+      <c r="I31" s="2" t="s">
+        <v>167</v>
+      </c>
+      <c r="J31" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="K31" s="2" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="32" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="2" t="s">
+        <v>169</v>
+      </c>
+      <c r="B32" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C32" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D32" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="E32" s="2" t="s">
+        <v>170</v>
+      </c>
+      <c r="F32" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="G32" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="H32" s="2" t="s">
+        <v>171</v>
+      </c>
+      <c r="I32" s="2" t="s">
+        <v>172</v>
+      </c>
+      <c r="J32" s="2" t="s">
+        <v>173</v>
+      </c>
+      <c r="K32" s="2" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="33" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A33" s="2" t="s">
+        <v>174</v>
+      </c>
+      <c r="B33" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C33" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D33" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E33" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="F33" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="G33" s="2" t="s">
+        <v>176</v>
+      </c>
+      <c r="H33" s="2" t="s">
+        <v>177</v>
+      </c>
+      <c r="I33" s="2" t="s">
+        <v>178</v>
+      </c>
+      <c r="J33" s="2" t="s">
+        <v>179</v>
+      </c>
+      <c r="K33" s="2" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="34" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A34" s="2" t="s">
+        <v>180</v>
+      </c>
+      <c r="B34" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C34" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D34" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="E34" s="2" t="s">
+        <v>181</v>
+      </c>
+      <c r="F34" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="G34" s="2" t="s">
+        <v>176</v>
+      </c>
+      <c r="H34" s="2" t="s">
+        <v>182</v>
+      </c>
+      <c r="I34" s="2" t="s">
+        <v>183</v>
+      </c>
+      <c r="J34" s="2" t="s">
+        <v>184</v>
+      </c>
+      <c r="K34" s="2" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="35" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A35" s="2" t="s">
+        <v>185</v>
+      </c>
+      <c r="B35" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C35" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D35" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="E35" s="2" t="s">
+        <v>186</v>
+      </c>
+      <c r="F35" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="G35" s="2" t="s">
+        <v>176</v>
+      </c>
+      <c r="H35" s="2" t="s">
+        <v>187</v>
+      </c>
+      <c r="I35" s="2" t="s">
+        <v>188</v>
+      </c>
+      <c r="J35" s="2" t="s">
+        <v>189</v>
+      </c>
+      <c r="K35" s="2" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="36" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A36" s="2" t="s">
+        <v>190</v>
+      </c>
+      <c r="B36" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C36" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D36" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="E36" s="2" t="s">
+        <v>191</v>
+      </c>
+      <c r="F36" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="G36" s="2" t="s">
+        <v>176</v>
+      </c>
+      <c r="H36" s="2" t="s">
+        <v>192</v>
+      </c>
+      <c r="I36" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="J36" s="2" t="s">
+        <v>194</v>
+      </c>
+      <c r="K36" s="2" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="37" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A37" s="2" t="s">
+        <v>195</v>
+      </c>
+      <c r="B37" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C37" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D37" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="E37" s="2" t="s">
+        <v>196</v>
+      </c>
+      <c r="F37" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="G37" s="2" t="s">
+        <v>176</v>
+      </c>
+      <c r="H37" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="I37" s="2" t="s">
+        <v>198</v>
+      </c>
+      <c r="J37" s="2" t="s">
+        <v>199</v>
+      </c>
+      <c r="K37" s="2" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="38" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A38" s="2" t="s">
+        <v>200</v>
+      </c>
+      <c r="B38" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C38" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D38" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="E38" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="F38" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="G38" s="2" t="s">
+        <v>176</v>
+      </c>
+      <c r="H38" s="2" t="s">
+        <v>202</v>
+      </c>
+      <c r="I38" s="2" t="s">
+        <v>203</v>
+      </c>
+      <c r="J38" s="2" t="s">
+        <v>204</v>
+      </c>
+      <c r="K38" s="2" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="39" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A39" s="2" t="s">
+        <v>205</v>
+      </c>
+      <c r="B39" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C39" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D39" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="E39" s="2" t="s">
+        <v>206</v>
+      </c>
+      <c r="F39" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="G39" s="2" t="s">
+        <v>176</v>
+      </c>
+      <c r="H39" s="2" t="s">
+        <v>207</v>
+      </c>
+      <c r="I39" s="2" t="s">
+        <v>208</v>
+      </c>
+      <c r="J39" s="2" t="s">
+        <v>209</v>
+      </c>
+      <c r="K39" s="2" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="40" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A40" s="2" t="s">
+        <v>210</v>
+      </c>
+      <c r="B40" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C40" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D40" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="E40" s="2" t="s">
+        <v>211</v>
+      </c>
+      <c r="F40" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="G40" s="2" t="s">
+        <v>176</v>
+      </c>
+      <c r="H40" s="2" t="s">
+        <v>212</v>
+      </c>
+      <c r="I40" s="2" t="s">
+        <v>213</v>
+      </c>
+      <c r="J40" s="2" t="s">
+        <v>214</v>
+      </c>
+      <c r="K40" s="2" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="41" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A41" s="2" t="s">
+        <v>215</v>
+      </c>
+      <c r="B41" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C41" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D41" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="E41" s="2" t="s">
+        <v>216</v>
+      </c>
+      <c r="F41" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="G41" s="2" t="s">
+        <v>176</v>
+      </c>
+      <c r="H41" s="2" t="s">
+        <v>217</v>
+      </c>
+      <c r="I41" s="2" t="s">
+        <v>218</v>
+      </c>
+      <c r="J41" s="2" t="s">
+        <v>219</v>
+      </c>
+      <c r="K41" s="2" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="42" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A42" s="2" t="s">
+        <v>220</v>
+      </c>
+      <c r="B42" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C42" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D42" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="E42" s="2" t="s">
+        <v>221</v>
+      </c>
+      <c r="F42" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="G42" s="2" t="s">
+        <v>176</v>
+      </c>
+      <c r="H42" s="2" t="s">
+        <v>222</v>
+      </c>
+      <c r="I42" s="2" t="s">
+        <v>223</v>
+      </c>
+      <c r="J42" s="2" t="s">
+        <v>224</v>
+      </c>
+      <c r="K42" s="2" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="43" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A43" s="2" t="s">
+        <v>225</v>
+      </c>
+      <c r="B43" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C43" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D43" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="E43" s="2" t="s">
+        <v>226</v>
+      </c>
+      <c r="F43" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="G43" s="2" t="s">
+        <v>176</v>
+      </c>
+      <c r="H43" s="2" t="s">
+        <v>227</v>
+      </c>
+      <c r="I43" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="J43" s="2" t="s">
+        <v>229</v>
+      </c>
+      <c r="K43" s="2" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="44" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A44" s="2" t="s">
+        <v>230</v>
+      </c>
+      <c r="B44" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C44" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D44" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="E44" s="2" t="s">
+        <v>231</v>
+      </c>
+      <c r="F44" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="G44" s="2" t="s">
+        <v>176</v>
+      </c>
+      <c r="H44" s="2" t="s">
+        <v>232</v>
+      </c>
+      <c r="I44" s="2" t="s">
+        <v>233</v>
+      </c>
+      <c r="J44" s="2" t="s">
+        <v>234</v>
+      </c>
+      <c r="K44" s="2" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="45" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A45" s="2" t="s">
+        <v>235</v>
+      </c>
+      <c r="B45" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C45" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D45" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="E45" s="2" t="s">
+        <v>236</v>
+      </c>
+      <c r="F45" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="G45" s="2" t="s">
+        <v>237</v>
+      </c>
+      <c r="H45" s="2" t="s">
+        <v>238</v>
+      </c>
+      <c r="I45" s="2" t="s">
+        <v>239</v>
+      </c>
+      <c r="J45" s="2" t="s">
+        <v>240</v>
+      </c>
+      <c r="K45" s="2" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="46" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A46" s="2" t="s">
+        <v>242</v>
+      </c>
+      <c r="B46" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C46" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D46" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="E46" s="2" t="s">
+        <v>243</v>
+      </c>
+      <c r="F46" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="G46" s="2" t="s">
+        <v>237</v>
+      </c>
+      <c r="H46" s="2" t="s">
+        <v>244</v>
+      </c>
+      <c r="I46" s="2" t="s">
+        <v>245</v>
+      </c>
+      <c r="J46" s="2" t="s">
+        <v>246</v>
+      </c>
+      <c r="K46" s="2" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="47" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A47" s="2" t="s">
+        <v>247</v>
+      </c>
+      <c r="B47" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C47" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D47" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="E47" s="2" t="s">
+        <v>248</v>
+      </c>
+      <c r="F47" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="G47" s="2" t="s">
+        <v>237</v>
+      </c>
+      <c r="H47" s="2" t="s">
+        <v>249</v>
+      </c>
+      <c r="I47" s="2" t="s">
+        <v>250</v>
+      </c>
+      <c r="J47" s="2" t="s">
+        <v>251</v>
+      </c>
+      <c r="K47" s="2" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="48" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A48" s="2" t="s">
+        <v>252</v>
+      </c>
+      <c r="B48" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C48" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D48" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="E48" s="2" t="s">
+        <v>253</v>
+      </c>
+      <c r="F48" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="G48" s="2" t="s">
+        <v>237</v>
+      </c>
+      <c r="H48" s="2" t="s">
+        <v>254</v>
+      </c>
+      <c r="I48" s="2" t="s">
+        <v>255</v>
+      </c>
+      <c r="J48" s="2" t="s">
+        <v>256</v>
+      </c>
+      <c r="K48" s="2" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="49" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A49" s="2" t="s">
+        <v>257</v>
+      </c>
+      <c r="B49" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C49" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D49" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="E49" s="2" t="s">
+        <v>258</v>
+      </c>
+      <c r="F49" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="G49" s="2" t="s">
+        <v>237</v>
+      </c>
+      <c r="H49" s="2" t="s">
+        <v>259</v>
+      </c>
+      <c r="I49" s="2" t="s">
+        <v>260</v>
+      </c>
+      <c r="J49" s="2" t="s">
+        <v>261</v>
+      </c>
+      <c r="K49" s="2" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="50" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A50" s="2" t="s">
+        <v>262</v>
+      </c>
+      <c r="B50" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C50" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D50" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="E50" s="2" t="s">
+        <v>263</v>
+      </c>
+      <c r="F50" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="G50" s="2" t="s">
+        <v>237</v>
+      </c>
+      <c r="H50" s="2" t="s">
+        <v>264</v>
+      </c>
+      <c r="I50" s="2" t="s">
+        <v>265</v>
+      </c>
+      <c r="J50" s="2" t="s">
+        <v>266</v>
+      </c>
+      <c r="K50" s="2" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="51" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A51" s="2" t="s">
+        <v>267</v>
+      </c>
+      <c r="B51" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C51" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D51" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="E51" s="2" t="s">
+        <v>268</v>
+      </c>
+      <c r="F51" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="G51" s="2" t="s">
+        <v>237</v>
+      </c>
+      <c r="H51" s="2" t="s">
+        <v>269</v>
+      </c>
+      <c r="I51" s="2" t="s">
+        <v>270</v>
+      </c>
+      <c r="J51" s="2" t="s">
+        <v>271</v>
+      </c>
+      <c r="K51" s="2" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="52" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A52" s="2" t="s">
+        <v>272</v>
+      </c>
+      <c r="B52" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C52" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D52" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="E52" s="2" t="s">
+        <v>273</v>
+      </c>
+      <c r="F52" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="G52" s="2" t="s">
+        <v>237</v>
+      </c>
+      <c r="H52" s="2" t="s">
+        <v>274</v>
+      </c>
+      <c r="I52" s="2" t="s">
+        <v>275</v>
+      </c>
+      <c r="J52" s="2" t="s">
+        <v>276</v>
+      </c>
+      <c r="K52" s="2" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="53" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A53" s="2" t="s">
+        <v>277</v>
+      </c>
+      <c r="B53" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C53" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D53" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="E53" s="2" t="s">
+        <v>278</v>
+      </c>
+      <c r="F53" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="G53" s="2" t="s">
+        <v>279</v>
+      </c>
+      <c r="H53" s="2" t="s">
+        <v>280</v>
+      </c>
+      <c r="I53" s="2" t="s">
+        <v>281</v>
+      </c>
+      <c r="J53" s="2" t="s">
+        <v>282</v>
+      </c>
+      <c r="K53" s="2" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="54" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A54" s="2" t="s">
+        <v>284</v>
+      </c>
+      <c r="B54" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C54" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D54" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="E54" s="2" t="s">
+        <v>285</v>
+      </c>
+      <c r="F54" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="G54" s="2" t="s">
+        <v>286</v>
+      </c>
+      <c r="H54" s="2" t="s">
+        <v>287</v>
+      </c>
+      <c r="I54" s="2" t="s">
+        <v>288</v>
+      </c>
+      <c r="J54" s="2" t="s">
+        <v>289</v>
+      </c>
+      <c r="K54" s="2" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="55" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A55" s="2" t="s">
+        <v>290</v>
+      </c>
+      <c r="B55" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C55" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D55" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="E55" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="F55" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="G55" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="H55" s="2" t="s">
+        <v>291</v>
+      </c>
+      <c r="I55" s="2" t="s">
+        <v>292</v>
+      </c>
+      <c r="J55" s="2" t="s">
+        <v>293</v>
+      </c>
+      <c r="K55" s="2" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="56" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A56" s="2" t="s">
+        <v>294</v>
+      </c>
+      <c r="B56" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C56" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D56" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="E56" s="2" t="s">
+        <v>160</v>
+      </c>
+      <c r="F56" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="G56" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="H56" s="2" t="s">
+        <v>295</v>
+      </c>
+      <c r="I56" s="2" t="s">
+        <v>296</v>
+      </c>
+      <c r="J56" s="2" t="s">
+        <v>297</v>
+      </c>
+      <c r="K56" s="2" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="57" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A57" s="2" t="s">
+        <v>298</v>
+      </c>
+      <c r="B57" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C57" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D57" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="E57" s="2" t="s">
+        <v>170</v>
+      </c>
+      <c r="F57" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="G57" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="H57" s="2" t="s">
+        <v>299</v>
+      </c>
+      <c r="I57" s="2" t="s">
+        <v>300</v>
+      </c>
+      <c r="J57" s="2" t="s">
+        <v>301</v>
+      </c>
+      <c r="K57" s="2" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="58" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A58" s="2" t="s">
+        <v>302</v>
+      </c>
+      <c r="B58" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C58" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D58" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="E58" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="F58" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="G58" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="H58" s="2" t="s">
+        <v>303</v>
+      </c>
+      <c r="I58" s="2" t="s">
+        <v>304</v>
+      </c>
+      <c r="J58" s="2" t="s">
+        <v>305</v>
+      </c>
+      <c r="K58" s="2" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="59" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A59" s="2" t="s">
+        <v>306</v>
+      </c>
+      <c r="B59" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C59" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D59" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="E59" s="2" t="s">
+        <v>253</v>
+      </c>
+      <c r="F59" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="G59" s="2" t="s">
+        <v>237</v>
+      </c>
+      <c r="H59" s="2" t="s">
+        <v>307</v>
+      </c>
+      <c r="I59" s="2" t="s">
+        <v>308</v>
+      </c>
+      <c r="J59" s="2" t="s">
+        <v>309</v>
+      </c>
+      <c r="K59" s="2" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="60" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A60" s="2" t="s">
+        <v>310</v>
+      </c>
+      <c r="B60" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C60" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D60" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="E60" s="2" t="s">
+        <v>258</v>
+      </c>
+      <c r="F60" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="G60" s="2" t="s">
+        <v>237</v>
+      </c>
+      <c r="H60" s="2" t="s">
+        <v>311</v>
+      </c>
+      <c r="I60" s="2" t="s">
+        <v>312</v>
+      </c>
+      <c r="J60" s="2" t="s">
+        <v>313</v>
+      </c>
+      <c r="K60" s="2" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="61" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A61" s="2" t="s">
+        <v>314</v>
+      </c>
+      <c r="B61" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C61" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D61" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="E61" s="2" t="s">
+        <v>268</v>
+      </c>
+      <c r="F61" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="G61" s="2" t="s">
+        <v>237</v>
+      </c>
+      <c r="H61" s="2" t="s">
+        <v>315</v>
+      </c>
+      <c r="I61" s="2" t="s">
+        <v>316</v>
+      </c>
+      <c r="J61" s="2" t="s">
+        <v>317</v>
+      </c>
+      <c r="K61" s="2" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="62" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A62" s="2" t="s">
+        <v>318</v>
+      </c>
+      <c r="B62" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C62" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D62" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="E62" s="2" t="s">
+        <v>273</v>
+      </c>
+      <c r="F62" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="G62" s="2" t="s">
+        <v>319</v>
+      </c>
+      <c r="H62" s="2" t="s">
+        <v>320</v>
+      </c>
+      <c r="I62" s="2" t="s">
+        <v>275</v>
+      </c>
+      <c r="J62" s="2" t="s">
+        <v>321</v>
+      </c>
+      <c r="K62" s="2" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="63" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A63" s="2" t="s">
+        <v>322</v>
+      </c>
+      <c r="B63" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C63" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D63" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E63" s="2" t="s">
+        <v>323</v>
+      </c>
+      <c r="F63" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="G63" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="H63" s="2" t="s">
+        <v>324</v>
+      </c>
+      <c r="I63" s="2" t="s">
+        <v>325</v>
+      </c>
+      <c r="J63" s="2" t="s">
+        <v>326</v>
+      </c>
+      <c r="K63" s="2" t="s">
+        <v>327</v>
+      </c>
+    </row>
+    <row r="64" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A64" s="2" t="s">
+        <v>328</v>
+      </c>
+      <c r="B64" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C64" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D64" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E64" s="2" t="s">
+        <v>329</v>
+      </c>
+      <c r="F64" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="G64" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="H64" s="2" t="s">
+        <v>330</v>
+      </c>
+      <c r="I64" s="2" t="s">
+        <v>331</v>
+      </c>
+      <c r="J64" s="2" t="s">
+        <v>332</v>
+      </c>
+      <c r="K64" s="2" t="s">
+        <v>327</v>
+      </c>
+    </row>
+    <row r="65" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A65" s="2" t="s">
+        <v>333</v>
+      </c>
+      <c r="B65" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C65" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D65" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="E65" s="2" t="s">
+        <v>334</v>
+      </c>
+      <c r="F65" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="G65" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="H65" s="2" t="s">
+        <v>335</v>
+      </c>
+      <c r="I65" s="2" t="s">
+        <v>336</v>
+      </c>
+      <c r="J65" s="2" t="s">
+        <v>337</v>
+      </c>
+      <c r="K65" s="2" t="s">
+        <v>327</v>
+      </c>
+    </row>
+    <row r="66" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A66" s="2" t="s">
+        <v>338</v>
+      </c>
+      <c r="B66" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C66" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D66" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="E66" s="2" t="s">
+        <v>339</v>
+      </c>
+      <c r="F66" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="G66" s="2" t="s">
+        <v>286</v>
+      </c>
+      <c r="H66" s="2" t="s">
+        <v>340</v>
+      </c>
+      <c r="I66" s="2" t="s">
+        <v>341</v>
+      </c>
+      <c r="J66" s="2" t="s">
+        <v>342</v>
+      </c>
+      <c r="K66" s="2" t="s">
+        <v>327</v>
+      </c>
+    </row>
+    <row r="67" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A67" s="2" t="s">
+        <v>343</v>
+      </c>
+      <c r="B67" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C67" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D67" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="E67" s="2" t="s">
+        <v>344</v>
+      </c>
+      <c r="F67" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="G67" s="2" t="s">
+        <v>286</v>
+      </c>
+      <c r="H67" s="2" t="s">
+        <v>345</v>
+      </c>
+      <c r="I67" s="2" t="s">
+        <v>346</v>
+      </c>
+      <c r="J67" s="2" t="s">
+        <v>347</v>
+      </c>
+      <c r="K67" s="2" t="s">
+        <v>327</v>
+      </c>
+    </row>
+    <row r="68" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A68" s="2" t="s">
+        <v>348</v>
+      </c>
+      <c r="B68" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C68" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D68" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="E68" s="2" t="s">
+        <v>349</v>
+      </c>
+      <c r="F68" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="G68" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="H68" s="2" t="s">
+        <v>350</v>
+      </c>
+      <c r="I68" s="2" t="s">
+        <v>351</v>
+      </c>
+      <c r="J68" s="2" t="s">
+        <v>352</v>
+      </c>
+      <c r="K68" s="2" t="s">
+        <v>327</v>
+      </c>
+    </row>
+    <row r="69" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A69" s="2" t="s">
+        <v>353</v>
+      </c>
+      <c r="B69" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C69" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D69" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="E69" s="2" t="s">
+        <v>354</v>
+      </c>
+      <c r="F69" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="G69" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="H69" s="2" t="s">
+        <v>355</v>
+      </c>
+      <c r="I69" s="2" t="s">
+        <v>356</v>
+      </c>
+      <c r="J69" s="2" t="s">
+        <v>357</v>
+      </c>
+      <c r="K69" s="2" t="s">
+        <v>327</v>
+      </c>
+    </row>
+    <row r="70" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A70" s="2" t="s">
+        <v>358</v>
+      </c>
+      <c r="B70" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C70" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D70" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="E70" s="2" t="s">
+        <v>359</v>
+      </c>
+      <c r="F70" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="G70" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="H70" s="2" t="s">
+        <v>360</v>
+      </c>
+      <c r="I70" s="2" t="s">
+        <v>361</v>
+      </c>
+      <c r="J70" s="2" t="s">
+        <v>362</v>
+      </c>
+      <c r="K70" s="2" t="s">
+        <v>327</v>
+      </c>
+    </row>
+    <row r="71" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A71" s="2" t="s">
+        <v>363</v>
+      </c>
+      <c r="B71" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C71" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D71" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="E71" s="2" t="s">
+        <v>364</v>
+      </c>
+      <c r="F71" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="G71" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="H71" s="2" t="s">
+        <v>365</v>
+      </c>
+      <c r="I71" s="2" t="s">
+        <v>366</v>
+      </c>
+      <c r="J71" s="2" t="s">
+        <v>367</v>
+      </c>
+      <c r="K71" s="2" t="s">
+        <v>327</v>
+      </c>
+    </row>
+    <row r="72" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A72" s="2" t="s">
+        <v>368</v>
+      </c>
+      <c r="B72" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C72" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D72" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="E72" s="2" t="s">
+        <v>369</v>
+      </c>
+      <c r="F72" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="G72" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="H72" s="2" t="s">
+        <v>370</v>
+      </c>
+      <c r="I72" s="2" t="s">
+        <v>371</v>
+      </c>
+      <c r="J72" s="2" t="s">
+        <v>372</v>
+      </c>
+      <c r="K72" s="2" t="s">
+        <v>327</v>
+      </c>
+    </row>
+    <row r="73" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A73" s="2" t="s">
+        <v>373</v>
+      </c>
+      <c r="B73" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C73" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D73" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="E73" s="2" t="s">
+        <v>374</v>
+      </c>
+      <c r="F73" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="G73" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="H73" s="2" t="s">
+        <v>375</v>
+      </c>
+      <c r="I73" s="2" t="s">
+        <v>376</v>
+      </c>
+      <c r="J73" s="2" t="s">
+        <v>377</v>
+      </c>
+      <c r="K73" s="2" t="s">
+        <v>327</v>
+      </c>
+    </row>
+    <row r="74" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A74" s="2" t="s">
+        <v>378</v>
+      </c>
+      <c r="B74" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C74" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D74" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="E74" s="2" t="s">
+        <v>379</v>
+      </c>
+      <c r="F74" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="G74" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="H74" s="2" t="s">
+        <v>380</v>
+      </c>
+      <c r="I74" s="2" t="s">
+        <v>381</v>
+      </c>
+      <c r="J74" s="2" t="s">
+        <v>382</v>
+      </c>
+      <c r="K74" s="2" t="s">
+        <v>327</v>
+      </c>
+    </row>
+    <row r="75" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A75" s="2" t="s">
+        <v>383</v>
+      </c>
+      <c r="B75" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C75" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D75" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="E75" s="2" t="s">
+        <v>384</v>
+      </c>
+      <c r="F75" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="G75" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="H75" s="2" t="s">
+        <v>385</v>
+      </c>
+      <c r="I75" s="2" t="s">
+        <v>386</v>
+      </c>
+      <c r="J75" s="2" t="s">
+        <v>387</v>
+      </c>
+      <c r="K75" s="2" t="s">
+        <v>327</v>
+      </c>
+    </row>
+    <row r="76" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A76" s="2" t="s">
+        <v>388</v>
+      </c>
+      <c r="B76" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C76" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D76" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="E76" s="2" t="s">
+        <v>389</v>
+      </c>
+      <c r="F76" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="G76" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="H76" s="2" t="s">
+        <v>390</v>
+      </c>
+      <c r="I76" s="2" t="s">
+        <v>391</v>
+      </c>
+      <c r="J76" s="2" t="s">
+        <v>392</v>
+      </c>
+      <c r="K76" s="2" t="s">
+        <v>327</v>
+      </c>
+    </row>
+    <row r="77" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A77" s="2" t="s">
+        <v>393</v>
+      </c>
+      <c r="B77" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C77" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D77" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="E77" s="2" t="s">
+        <v>394</v>
+      </c>
+      <c r="F77" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="G77" s="2" t="s">
+        <v>395</v>
+      </c>
+      <c r="H77" s="2" t="s">
+        <v>396</v>
+      </c>
+      <c r="I77" s="2" t="s">
+        <v>397</v>
+      </c>
+      <c r="J77" s="2" t="s">
+        <v>398</v>
+      </c>
+      <c r="K77" s="2" t="s">
+        <v>327</v>
+      </c>
+    </row>
+    <row r="78" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A78" s="2" t="s">
+        <v>399</v>
+      </c>
+      <c r="B78" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C78" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D78" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E78" s="2" t="s">
+        <v>400</v>
+      </c>
+      <c r="F78" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="G78" s="2" t="s">
+        <v>237</v>
+      </c>
+      <c r="H78" s="2" t="s">
+        <v>401</v>
+      </c>
+      <c r="I78" s="2" t="s">
+        <v>402</v>
+      </c>
+      <c r="J78" s="2" t="s">
+        <v>403</v>
+      </c>
+      <c r="K78" s="2" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="79" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A79" s="2" t="s">
+        <v>405</v>
+      </c>
+      <c r="B79" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C79" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D79" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="E79" s="2" t="s">
+        <v>406</v>
+      </c>
+      <c r="F79" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="G79" s="2" t="s">
+        <v>176</v>
+      </c>
+      <c r="H79" s="2" t="s">
+        <v>407</v>
+      </c>
+      <c r="I79" s="2" t="s">
+        <v>408</v>
+      </c>
+      <c r="J79" s="2" t="s">
+        <v>409</v>
+      </c>
+      <c r="K79" s="2" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="80" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A80" s="2" t="s">
+        <v>410</v>
+      </c>
+      <c r="B80" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C80" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D80" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="E80" s="2" t="s">
+        <v>411</v>
+      </c>
+      <c r="F80" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="G80" s="2" t="s">
+        <v>412</v>
+      </c>
+      <c r="H80" s="2" t="s">
+        <v>413</v>
+      </c>
+      <c r="I80" s="2" t="s">
+        <v>414</v>
+      </c>
+      <c r="J80" s="2" t="s">
+        <v>415</v>
+      </c>
+      <c r="K80" s="2" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="81" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A81" s="2" t="s">
+        <v>416</v>
+      </c>
+      <c r="B81" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C81" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D81" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="E81" s="2" t="s">
+        <v>417</v>
+      </c>
+      <c r="F81" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="G81" s="2" t="s">
+        <v>237</v>
+      </c>
+      <c r="H81" s="2" t="s">
+        <v>418</v>
+      </c>
+      <c r="I81" s="2" t="s">
+        <v>419</v>
+      </c>
+      <c r="J81" s="2" t="s">
+        <v>420</v>
+      </c>
+      <c r="K81" s="2" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="82" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A82" s="2" t="s">
+        <v>421</v>
+      </c>
+      <c r="B82" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C82" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D82" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="E82" s="2" t="s">
+        <v>422</v>
+      </c>
+      <c r="F82" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="G82" s="2" t="s">
+        <v>237</v>
+      </c>
+      <c r="H82" s="2" t="s">
+        <v>423</v>
+      </c>
+      <c r="I82" s="2" t="s">
+        <v>424</v>
+      </c>
+      <c r="J82" s="2" t="s">
+        <v>425</v>
+      </c>
+      <c r="K82" s="2" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="83" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A83" s="2" t="s">
+        <v>426</v>
+      </c>
+      <c r="B83" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C83" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D83" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="E83" s="2" t="s">
+        <v>427</v>
+      </c>
+      <c r="F83" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="G83" s="2" t="s">
+        <v>237</v>
+      </c>
+      <c r="H83" s="2" t="s">
+        <v>428</v>
+      </c>
+      <c r="I83" s="2" t="s">
+        <v>429</v>
+      </c>
+      <c r="J83" s="2" t="s">
+        <v>430</v>
+      </c>
+      <c r="K83" s="2" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="84" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A84" s="2" t="s">
+        <v>431</v>
+      </c>
+      <c r="B84" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C84" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D84" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="E84" s="2" t="s">
+        <v>432</v>
+      </c>
+      <c r="F84" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="G84" s="2" t="s">
+        <v>237</v>
+      </c>
+      <c r="H84" s="2" t="s">
+        <v>433</v>
+      </c>
+      <c r="I84" s="2" t="s">
+        <v>434</v>
+      </c>
+      <c r="J84" s="2" t="s">
+        <v>435</v>
+      </c>
+      <c r="K84" s="2" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="85" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A85" s="2" t="s">
+        <v>436</v>
+      </c>
+      <c r="B85" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C85" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D85" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="E85" s="2" t="s">
+        <v>437</v>
+      </c>
+      <c r="F85" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="G85" s="2" t="s">
+        <v>237</v>
+      </c>
+      <c r="H85" s="2" t="s">
+        <v>438</v>
+      </c>
+      <c r="I85" s="2" t="s">
+        <v>439</v>
+      </c>
+      <c r="J85" s="2" t="s">
+        <v>440</v>
+      </c>
+      <c r="K85" s="2" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="86" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A86" s="2" t="s">
+        <v>441</v>
+      </c>
+      <c r="B86" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C86" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D86" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="E86" s="2" t="s">
+        <v>442</v>
+      </c>
+      <c r="F86" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="G86" s="2" t="s">
+        <v>237</v>
+      </c>
+      <c r="H86" s="2" t="s">
+        <v>443</v>
+      </c>
+      <c r="I86" s="2" t="s">
+        <v>444</v>
+      </c>
+      <c r="J86" s="2" t="s">
+        <v>445</v>
+      </c>
+      <c r="K86" s="2" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="87" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A87" s="2" t="s">
+        <v>446</v>
+      </c>
+      <c r="B87" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C87" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D87" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="E87" s="2" t="s">
+        <v>447</v>
+      </c>
+      <c r="F87" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="G87" s="2" t="s">
+        <v>237</v>
+      </c>
+      <c r="H87" s="2" t="s">
+        <v>448</v>
+      </c>
+      <c r="I87" s="2" t="s">
+        <v>449</v>
+      </c>
+      <c r="J87" s="2" t="s">
+        <v>450</v>
+      </c>
+      <c r="K87" s="2" t="s">
+        <v>404</v>
+      </c>
+    </row>
   </sheetData>
-  <drawing r:id="rId1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
updated circulatory system data
</commit_message>
<xml_diff>
--- a/ai/data/raw/Project_CirculatorySystem_EDatas.xlsx
+++ b/ai/data/raw/Project_CirculatorySystem_EDatas.xlsx
@@ -151,7 +151,7 @@
     <t>Atrium sinister (sol kulakçık) kalbin sol üst odacığıdır.</t>
   </si>
   <si>
-    <t>["Akciğerlerden oksijen bakımından zengin kan akciğer toplardamarları aracılığıyla buraya gelir."  , "Sol kulakçık bu kanı mitral kapaktan geçirerek sol karıncığa iletir."]</t>
+    <t>["Akciğerlerden oksijen bakımından zengin kan V. pulmonales aracılığıyla buraya gelir."  , "Sol kulakçık bu kanı mitral kapaktan geçirerek sol karıncığa iletir."]</t>
   </si>
   <si>
     <t>ventriculus_dexter</t>
@@ -166,7 +166,7 @@
     <t>Ventriculus dexter (sağ karıncık) kalbin sağ alt odacığıdır.</t>
   </si>
   <si>
-    <t>["Sağ kulakçıktan gelen oksijeni azalmış kanı akciğerlere gönderir." , "Bu kan akciğer atardamarı aracılığıyla akciğerlere taşınır ve burada oksijenlenir."]</t>
+    <t>["Sağ kulakçıktan gelen oksijeni azalmış kanı akciğerlere gönderir." , "Bu kan A. pulmonalis aracılığıyla akciğerlere taşınır ve burada oksijenlenir."]</t>
   </si>
   <si>
     <t>ventriculus_sinister</t>
@@ -190,1230 +190,1233 @@
     <t>vessel</t>
   </si>
   <si>
-    <t>Üst ana toplardamar</t>
+    <t>Vena cava superior</t>
   </si>
   <si>
     <t>heart; vessel; vein</t>
   </si>
   <si>
-    <t>Üst ana toplardamar, baş ve üst vücut bölgelerinden gelen oksijeni azalmış kanı kalbin sağ kulakçığına taşıyan büyük toplardamardır.</t>
+    <t>Vena cava superior,  baş ve üst vücut bölgelerinden gelen oksijeni azalmış kanı kalbin sağ kulakçığına taşıyan büyük toplardamardır.</t>
   </si>
   <si>
     <t>vena_cava_inferior</t>
   </si>
   <si>
-    <t>Alt ana toplardamar</t>
-  </si>
-  <si>
-    <t>Alt ana toplardamar, vücudun alt bölgelerinden gelen oksijeni azalmış kanı kalbin sağ kulakçığına taşıyan büyük toplardamardır.</t>
+    <t>Vena cava inferior</t>
+  </si>
+  <si>
+    <t>Vena cava inferior, vücudun alt bölgelerinden gelen oksijeni azalmış kanı kalbin sağ kulakçığına taşıyan büyük toplardamardır.</t>
   </si>
   <si>
     <t>aorta</t>
   </si>
   <si>
+    <t>Aorta</t>
+  </si>
+  <si>
+    <t>heart; vessel; artery; aorta</t>
+  </si>
+  <si>
+    <t>Aort, kalpten çıkan en büyük atardamardır.</t>
+  </si>
+  <si>
+    <t>["Sol karıncıktan çıkan oksijen bakımından zengin kanı tüm vücuda taşır." , "Aort, sistemik dolaşımın başlangıç damarıdır."]</t>
+  </si>
+  <si>
+    <t>pulmonary_vein</t>
+  </si>
+  <si>
+    <t>V. pulmonales</t>
+  </si>
+  <si>
+    <t>heart; vessel; vein; pulmonary</t>
+  </si>
+  <si>
+    <t>V. pulmonales, akciğerlerde oksijenlenen kanı kalbin sol kulakçığına taşıyan damarlardır.</t>
+  </si>
+  <si>
+    <t>["Akciğerlerden gelen oksijen bakımından zengin kanı kalbe getirir.", "Diğer toplardamarlardan farklı olarak oksijen bakımından zengin kan taşır."]</t>
+  </si>
+  <si>
+    <t>heart_valves</t>
+  </si>
+  <si>
+    <t>Kalbin kapakları</t>
+  </si>
+  <si>
+    <t>heart; valve; mitral; tricuspid; aortic; pulmonary</t>
+  </si>
+  <si>
+    <t>Kalpte dört adet kapak bulunur.</t>
+  </si>
+  <si>
+    <t>["Bu kapakların ikisi atriyoventriküler kapaklar, ikisi ise semilunar kapaklardır." , "Atriyoventriküler kapaklar, kulakçıklar ile karıncıklar arasında yer alır ve mitral kapak ile triküspit kapaktan oluşur." , "Semilunar kapaklar ise karıncıklar ile büyük atardamarlar arasında bulunur ve aort kapağı ile pulmoner kapaktan oluşur.", "Kalp kapakları, kalbin kasılması ve gevşemesi sırasında kanın geriye doğru akmasını engelleyerek kanın tek yönlü ilerlemesini sağlar."]</t>
+  </si>
+  <si>
+    <t>Ders kitabı s.132</t>
+  </si>
+  <si>
+    <t>coronary_arteries</t>
+  </si>
+  <si>
+    <t>Koroner arterler</t>
+  </si>
+  <si>
+    <t>heart; coronary; artery; circulation</t>
+  </si>
+  <si>
+    <t>Kalp kasına oksijen bakımından zengin kan taşıyan damarlara koroner arterler denir.</t>
+  </si>
+  <si>
+    <t>["Koroner arterler aorttan ayrılan ilk dallardır." , "Sağ koroner arter kalbin sağ tarafını, sol koroner arter ise kalbin sol tarafını besler." , "Bu damarlarda oluşan daralma veya tıkanıklıklar kalp kasının yeterince beslenmesini engelleyebilir ve kalp krizine neden olabilir."]</t>
+  </si>
+  <si>
+    <t>arteria_coronalis_dextra</t>
+  </si>
+  <si>
+    <t>Arteria coronalis dextra</t>
+  </si>
+  <si>
+    <t>heart; coronary; artery; right</t>
+  </si>
+  <si>
+    <t>Sağ koroner arter (arteria coronalis dextra), aorttan ayrılan ve kalbin sağ tarafını besleyen koroner damardır.</t>
+  </si>
+  <si>
+    <t>["Aorttan ayrılan ilk dallardan biridir.", "Kalp kasına oksijen ve besin bakımından zengin kan taşır."]</t>
+  </si>
+  <si>
+    <t>arteria_coronalis_sinistra</t>
+  </si>
+  <si>
+    <t>Arteria coronalis sinistra</t>
+  </si>
+  <si>
+    <t>heart; coronary; artery; left</t>
+  </si>
+  <si>
+    <t>Sol koroner arter (arteria coronalis sinistra), aorttan ayrılan ve kalbin sol tarafını besleyen koroner damardır.</t>
+  </si>
+  <si>
+    <t>["Kalp kasının büyük bölümüne oksijen bakımından zengin kan taşır."]</t>
+  </si>
+  <si>
+    <t>vena_cordis_magna</t>
+  </si>
+  <si>
+    <t>Vena cordis magna</t>
+  </si>
+  <si>
+    <t>heart; coronary; vein</t>
+  </si>
+  <si>
+    <t>Vena cordis magna, kalp kasından toplanan kirli kanı taşıyan büyük koroner toplardamarlardan biridir.</t>
+  </si>
+  <si>
+    <t>["Bu damar kalbin yüzeyindeki venlerle birleşerek koroner sinüse katılır."]</t>
+  </si>
+  <si>
+    <t>vena_cordis_media</t>
+  </si>
+  <si>
+    <t>Vena cordis media</t>
+  </si>
+  <si>
+    <t>Vena cordis media, kalp kasından gelen kirli kanı toplayan koroner toplardamarlardan biridir.</t>
+  </si>
+  <si>
+    <t>["Bu damar da diğer koroner venlerle birlikte koroner sinüse açılır."]</t>
+  </si>
+  <si>
+    <t>vena_cordis_parva</t>
+  </si>
+  <si>
+    <t>Vena cordis parva</t>
+  </si>
+  <si>
+    <t>Vena cordis parva, kalp kasından gelen kirli kanı taşıyan küçük koroner toplardamarlardan biridir.</t>
+  </si>
+  <si>
+    <t>["Bu damar koroner venlerle birleşerek koroner sinüse katılır."]</t>
+  </si>
+  <si>
+    <t>coronary_sinus</t>
+  </si>
+  <si>
+    <t>Sinus coronarius</t>
+  </si>
+  <si>
+    <t>heart; coronary; sinus</t>
+  </si>
+  <si>
+    <t>Sinus coronarius, kalp kasından gelen kirli kanın toplandığı geniş bir toplardamardır.</t>
+  </si>
+  <si>
+    <t>["Koroner venler burada birleşir ve kan buradan sağ atriyuma dökülür."]</t>
+  </si>
+  <si>
+    <t>cardiac_cycle</t>
+  </si>
+  <si>
+    <t>Kalbin çalışması</t>
+  </si>
+  <si>
+    <t>heart; cardiac cycle; systole; diastole</t>
+  </si>
+  <si>
+    <t>Kalp, kendine ait uyarı çıkaran hücreler sayesinde düzenli olarak kasılıp gevşer.</t>
+  </si>
+  <si>
+    <t>["Kalbin kasılma evresine sistol, gevşeme evresine ise diyastol denir." , "Ventriküller kasıldığında kan atardamarlara pompalanır, gevşediğinde ise atriyumlardan gelen kan ventriküllere dolar." , "Kapaklar kanın tek yönlü ilerlemesini sağlar ve geri kaçmasını engeller."]</t>
+  </si>
+  <si>
+    <t>Ders kitabı s.134</t>
+  </si>
+  <si>
+    <t>tricuspid_valve</t>
+  </si>
+  <si>
+    <t>Triküspit kapak</t>
+  </si>
+  <si>
+    <t>heart; valve; tricuspid</t>
+  </si>
+  <si>
+    <t>Triküspit kapak, sağ kulakçık ile sağ karıncık arasında bulunan atriyoventriküler kapaktır.</t>
+  </si>
+  <si>
+    <t>["Ventrikül kasıldığında kanın tekrar kulakçığa geri dönmesini engeller."]</t>
+  </si>
+  <si>
+    <t>mitral_valve</t>
+  </si>
+  <si>
+    <t>Mitral kapak</t>
+  </si>
+  <si>
+    <t>heart; valve; mitral</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mitral kapak, sol kulakçık ile sol karıncık arasında bulunan atriyoventriküler kapaktır. </t>
+  </si>
+  <si>
+    <t>["Kanın ventrikül kasılması sırasında sol kulakçığa geri kaçmasını engeller."]</t>
+  </si>
+  <si>
+    <t>myocardium</t>
+  </si>
+  <si>
+    <t>Myocardium</t>
+  </si>
+  <si>
+    <t>heart; muscle; myocardium</t>
+  </si>
+  <si>
+    <t>Myokard, kalbin kasılmasını sağlayan kalın kas tabakasıdır.</t>
+  </si>
+  <si>
+    <t>["Bu kas tabakası kasılarak kanın kalpten damarlara pompalanmasını sağlar."]</t>
+  </si>
+  <si>
+    <t>arteries</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Arteriae  </t>
+  </si>
+  <si>
+    <t>Vessels</t>
+  </si>
+  <si>
+    <t>artery; arter; vessel; blood circulation; damar</t>
+  </si>
+  <si>
+    <t>Atardamarlar, kanı kalpten dokulara ve organlara taşıyan kan damarlarıdır.</t>
+  </si>
+  <si>
+    <t>["Arterler kalbin ventrikülleri ile bağlantılı damarlardır ve kanı kalpten uzaklaştırarak vücudun farklı bölgelerine taşırlar.", "Sağ ventrikülden akciğerlere kirli kan taşıyan A. pulmonalis dışında diğer tüm atardamarlar oksijen bakımından zengin temiz kan taşır.", "Sol ventrikülden çıkan temiz kan sistol sırasında aort damarına pompalanır ve buradan vücuttaki diğer atardamarlara dağıtılır.", "Arterlerin çapları perifer bölgelere doğru gidildikçe küçülür ve bu küçük damarlara arteriyol adı verilir.", "Arterlerde kan basıncı yüksek olduğu için damar duvarları toplardamarlara göre daha kalın ve dayanıklıdır."]</t>
+  </si>
+  <si>
+    <t>Ders kitabı s.138</t>
+  </si>
+  <si>
+    <t>upper_extremity_arteries</t>
+  </si>
+  <si>
+    <t>Üst ekstremite arterleri</t>
+  </si>
+  <si>
+    <t>Upper_Extremity</t>
+  </si>
+  <si>
+    <t>artery; arter; upper extremity; arm; kol; damar; subclavian; axillary; brachial; radial; ulnar</t>
+  </si>
+  <si>
+    <t>Üst ekstremite arterleri, omuzdan ele kadar üst ekstremiteyi besleyen atardamarlardır.</t>
+  </si>
+  <si>
+    <t>["Sağ ve sol köprücük altı arterleri kola doğru ilerledikçe çapları giderek küçülür ve geçtikleri bölgeye göre farklı isimler alırlar.","Üst ekstremitede arterler sırasıyla a. subclavia, a. axillaris, a. brachialis, a. radialis ve a. ulnaris olarak devam eder.","Bu damarlar omuz, kol, ön kol ve elin kanlanmasını sağlar."]</t>
+  </si>
+  <si>
+    <t>subclavian_artery</t>
+  </si>
+  <si>
+    <t>A. subclavia</t>
+  </si>
+  <si>
+    <t>artery; subclavian artery; a. subclavia; upper extremity; arter; köprücük altı atardamarı; atardamar</t>
+  </si>
+  <si>
+    <t>A. subclavia, üst ekstremiteye kan taşıyan ana arterlerden biridir.</t>
+  </si>
+  <si>
+    <t>["Sağ ve sol a. subclavia, üst ekstremiteye uzanan arteriyel dolaşımın başlangıç bölümünü oluşturur.","Bu damar kola doğru ilerledikçe bulunduğu bölgeye göre isim değiştirir.","Koltuk altı bölgesine ulaştığında a. axillaris adını alır."]</t>
+  </si>
+  <si>
+    <t>axillary_artery</t>
+  </si>
+  <si>
+    <t>A. axillaris</t>
+  </si>
+  <si>
+    <t>artery; arter; axillary artery; a. axillaris; koltuk altı atardamarı; upper extremity; atardamar</t>
+  </si>
+  <si>
+    <t>A. axillaris, a. subclavia'nın koltuk altı bölgesindeki devamıdır.</t>
+  </si>
+  <si>
+    <t>["A. subclavia, koltuk altı bölgesine geldiğinde a. axillaris adını alır.","A. axillaris göğüs ve omuz bölgesine dallar verir.","Bu damar kol bölgesine doğru devam ederek a. brachialis adını alır."]</t>
+  </si>
+  <si>
+    <t>brachial_artery</t>
+  </si>
+  <si>
+    <t>A. brachialis</t>
+  </si>
+  <si>
+    <t>artery; arter; brachial artery; a. brachialis; kol atardamarı; blood pressure; atardamar</t>
+  </si>
+  <si>
+    <t>A. brachialis, a. axillaris'in kol bölgesindeki devamıdır.</t>
+  </si>
+  <si>
+    <t>["A. axillaris kol bölgesine geçince a. brachialis adını alır.","A. brachialis kol kaslarının beslenmesini sağlar.","Tansiyon ölçümü klinikte bu damar üzerinden yapılır.","Dirsek ön bölgesinde a. radialis ve a. ulnaris olmak üzere iki dala ayrılır."]</t>
+  </si>
+  <si>
+    <t>radial_artery</t>
+  </si>
+  <si>
+    <t>A. radialis</t>
+  </si>
+  <si>
+    <t>artery; arter; radial artery; a. radialis; radius; nabız; pulse; upper extremity; atardamar</t>
+  </si>
+  <si>
+    <t>A. radialis, a. brachialis'in dirsek ön bölgesinde ayrılan dallarından biridir.</t>
+  </si>
+  <si>
+    <t>["A. brachialis dirsek ön bölgesinde a. radialis ve a. ulnaris olarak iki dala ayrılır.","A. radialis ön kolun ve elin bir bölümünün kanlanmasına katkı sağlar.","A. radialis nabız almada daha sık tercih edilen damarlardan biridir."]</t>
+  </si>
+  <si>
+    <t>ulnar_artery</t>
+  </si>
+  <si>
+    <t>A. ulnaris</t>
+  </si>
+  <si>
+    <t>artery; arter; ulnar artery; a. ulnaris; ulna; upper extremity; atardamar</t>
+  </si>
+  <si>
+    <t>A. ulnaris, a. brachialis'in dirsek ön bölgesinde ayrılan dallarından biridir.</t>
+  </si>
+  <si>
+    <t>["A. brachialis dirsek ön bölgesinde iki ana dala ayrılır ve bunlardan biri a. ulnaris'tir.","A. ulnaris ön kolun ve elin bir bölümünün kanlanmasına katkı sağlar.","A. ulnaris, a. radialis ile birlikte el bileği ve elin beslenmesinde görev alır."]</t>
+  </si>
+  <si>
+    <t>abdominal_aorta</t>
+  </si>
+  <si>
+    <t>Karın aortu</t>
+  </si>
+  <si>
+    <t>Abdomen</t>
+  </si>
+  <si>
+    <t>artery; abdominal aorta; aorta abdominalis; circulation; abdomen; atardamar</t>
+  </si>
+  <si>
+    <t>Karın aortu, aortun diyaframdan sonra karın boşluğunda devam eden bölümüdür.</t>
+  </si>
+  <si>
+    <t>["Karın aortu diyaframdan başlayarak bel omurları boyunca aşağı doğru uzanır.","Bu damar karın bölgesindeki birçok organa kan taşıyan arterlerin çıktığı ana damardır.","Truncus coeliacus, a. mesenterica superior ve a. mesenterica inferior gibi önemli arterler karın aortundan ayrılır.","Karın aortu yaklaşık dördüncü bel omuru hizasında ikiye ayrılarak sağ ve sol a. iliaca communis arterlerini oluşturur."]</t>
+  </si>
+  <si>
+    <t>truncus_coeliacus</t>
+  </si>
+  <si>
+    <t>Truncus coeliacus</t>
+  </si>
+  <si>
+    <t>artery; truncus coeliacus; celiac trunk; abdominal aorta; atardamar</t>
+  </si>
+  <si>
+    <t>Truncus coeliacus, karın aortundan ayrılan ve üç ana dala ayrılan önemli bir arterdir.</t>
+  </si>
+  <si>
+    <t>["Truncus coeliacus karın aortundan ayrılır.","Bu damar üç ana dala ayrılarak karın bölgesindeki bazı organlara kan taşır.","Dalları mide, karaciğer ve dalak gibi organların beslenmesine katkı sağlar."]</t>
+  </si>
+  <si>
+    <t>gastrica_sinistra</t>
+  </si>
+  <si>
+    <t>A. gastrica sinistra</t>
+  </si>
+  <si>
+    <t>artery; gastrica sinistra; left gastric artery; stomach; atardamar</t>
+  </si>
+  <si>
+    <t>A. gastrica sinistra, mideyi besleyen arterlerden biridir.</t>
+  </si>
+  <si>
+    <t>["Bu damar karın aortundan çıkan truncus coeliacusun dallarından biridir.","Midenin üst kısmına kan taşır.","Mide duvarının beslenmesine katkı sağlar."]</t>
+  </si>
+  <si>
+    <t>hepatica_communis</t>
+  </si>
+  <si>
+    <t>A. hepatica communis</t>
+  </si>
+  <si>
+    <t>artery; hepatica communis; common hepatic artery; liver; atardamar</t>
+  </si>
+  <si>
+    <t>A. hepatica communis, karaciğeri besleyen önemli arterlerden biridir.</t>
+  </si>
+  <si>
+    <t>["Bu damar truncus coeliacusun ana dallarından biridir.","Karaciğere kan taşır.","Karaciğer dokusunun beslenmesinde görev alır."]</t>
+  </si>
+  <si>
+    <t>lienalis</t>
+  </si>
+  <si>
+    <t>A. lienalis</t>
+  </si>
+  <si>
+    <t>artery; lienalis; splenic artery; spleen; pancreas; atardamar</t>
+  </si>
+  <si>
+    <t>A. lienalis, dalak ve pankreası besleyen arterlerden biridir.</t>
+  </si>
+  <si>
+    <t>["Bu damar truncus coeliacusun dallarından biridir.","Dalak dokusuna kan taşır.","Pankreasın bir bölümünün beslenmesine katkı sağlar."]</t>
+  </si>
+  <si>
+    <t>mesenterica_superior</t>
+  </si>
+  <si>
+    <t>A. mesenterica superior</t>
+  </si>
+  <si>
+    <t>artery; mesenterica superior; superior mesenteric artery; intestine; atardamar</t>
+  </si>
+  <si>
+    <t>A. mesenterica superior, ince bağırsak ve kalın bağırsağın bir bölümünü besleyen arterdir.</t>
+  </si>
+  <si>
+    <t>["Bu damar karın aortundan ayrılır.","İnce bağırsağa kan taşır.","Kalın bağırsağın ilk yarısının beslenmesine katkı sağlar."]</t>
+  </si>
+  <si>
+    <t>mesenterica_inferior</t>
+  </si>
+  <si>
+    <t>A. mesenterica inferior</t>
+  </si>
+  <si>
+    <t>artery; mesenterica inferior; inferior mesenteric artery; intestine; atardamar</t>
+  </si>
+  <si>
+    <t>A. mesenterica inferior, kalın bağırsağın ikinci yarısını besleyen arterdir.</t>
+  </si>
+  <si>
+    <t>["Bu damar karın aortundan ayrılır.","Kalın bağırsağın alt bölümlerine kan taşır.","Sindirim sisteminin alt kısmının beslenmesinde görev alır."]</t>
+  </si>
+  <si>
+    <t>renalis</t>
+  </si>
+  <si>
+    <t>A. renalis</t>
+  </si>
+  <si>
+    <t>artery; renalis; renal artery; kidney; atardamar</t>
+  </si>
+  <si>
+    <t>A. renalis, böbreklere kan taşıyan büyük arterlerden biridir.</t>
+  </si>
+  <si>
+    <t>["Bu damar karın aortundan ayrılır.","Böbreklere oksijen bakımından zengin kan taşır.","Böbrek dokusunun beslenmesinde önemli rol oynar."]</t>
+  </si>
+  <si>
+    <t>gonadal_artery</t>
+  </si>
+  <si>
+    <t>A. testicularis / A. ovarica</t>
+  </si>
+  <si>
+    <t>artery; testicular artery; ovarian artery; gonadal artery; atardamar</t>
+  </si>
+  <si>
+    <t>A. testicularis ve A. ovarica, üreme organlarını besleyen arterlerdir.</t>
+  </si>
+  <si>
+    <t>["Bu damarlar karın aortundan ayrılır.","Erkeklerde testislerin kanlanmasını sağlar.","Kadınlarda yumurtalıkların beslenmesinde görev alır."]</t>
+  </si>
+  <si>
+    <t>lumbales</t>
+  </si>
+  <si>
+    <t>A. lumbales</t>
+  </si>
+  <si>
+    <t>artery; lumbales; lumbar artery; spine; atardamar</t>
+  </si>
+  <si>
+    <t>A. lumbales, bel bölgesindeki yapıları besleyen arterlerdir.</t>
+  </si>
+  <si>
+    <t>["Bu damarlar karın aortundan ayrılır.","Omurilik çevresindeki kas ve dokulara kan taşırlar.","Bel bölgesinin kanlanmasına katkı sağlarlar."]</t>
+  </si>
+  <si>
+    <t>sacralis_media</t>
+  </si>
+  <si>
+    <t>A. sacralis media</t>
+  </si>
+  <si>
+    <t>artery; sacralis media; sacral artery; sacrum; atardamar</t>
+  </si>
+  <si>
+    <t>A. sacralis media, sakrum bölgesini besleyen arterdir.</t>
+  </si>
+  <si>
+    <t>["Bu damar karın aortunun alt kısmından ayrılır.","Sakrum bölgesine kan taşır.","Pelvis bölgesindeki bazı yapıların beslenmesine katkı sağlar."]</t>
+  </si>
+  <si>
+    <t>phrenica_inferior</t>
+  </si>
+  <si>
+    <t>A. phrenica inferior</t>
+  </si>
+  <si>
+    <t>artery; phrenica inferior; inferior phrenic artery; diaphragm; atardamar</t>
+  </si>
+  <si>
+    <t>A. phrenica inferior, diyaframın alt kısmını besleyen arterlerden biridir.</t>
+  </si>
+  <si>
+    <t>["Bu damar karın aortundan ayrılır.","Diyaframın alt yüzüne kan taşır.","Diyafram kasının beslenmesinde görev alır."]</t>
+  </si>
+  <si>
+    <t>iliaca_communis</t>
+  </si>
+  <si>
+    <t>A. iliaca communis</t>
+  </si>
+  <si>
+    <t>Lower_Extremity</t>
+  </si>
+  <si>
+    <t>artery; iliaca communis; common iliac artery; pelvis; atardamar</t>
+  </si>
+  <si>
+    <t>A. iliaca communis, karın aortunun ikiye ayrılmasıyla oluşan büyük arterlerden biridir.</t>
+  </si>
+  <si>
+    <t>["Karın aortu yaklaşık dördüncü bel omuru hizasında ikiye ayrılarak sağ ve sol a. iliaca communis arterlerini oluşturur.","Bu arter pelvis bölgesine doğru ilerler.","Pelvis içinde a. iliaca interna ve a. iliaca externa olmak üzere iki ana dala ayrılır."]</t>
+  </si>
+  <si>
+    <t>Ders kitabı s.139</t>
+  </si>
+  <si>
+    <t>iliaca_interna</t>
+  </si>
+  <si>
+    <t>A. iliaca interna</t>
+  </si>
+  <si>
+    <t>artery; iliaca interna; internal iliac artery; pelvis; atardamar</t>
+  </si>
+  <si>
+    <t>A. iliaca interna, pelvis boşluğundaki organları besleyen arterdir.</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> ["Bu damar a. iliaca communis'in dallarından biridir.","Pelvis boşluğu içinde ilerler.","Mesane, rektum ve pelvis kasları gibi yapılara dallar vererek bu bölgelerin beslenmesini sağlar."]</t>
+  </si>
+  <si>
+    <t>iliaca_externa</t>
+  </si>
+  <si>
+    <t>A. iliaca externa</t>
+  </si>
+  <si>
+    <t>artery; iliaca externa; external iliac artery; leg; atardamar</t>
+  </si>
+  <si>
+    <t>A. iliaca externa, alt ekstremiteye kan taşıyan önemli arterlerden biridir.</t>
+  </si>
+  <si>
+    <t>["Bu damar a. iliaca communis'in iki ana dalından biridir.","Pelvis bölgesinden çıkarak bacaklara doğru ilerler.","Alt ekstremitenin kanlanmasını sağlayan arteriyel dolaşımın devamını oluşturur."]</t>
+  </si>
+  <si>
+    <t>femoralis</t>
+  </si>
+  <si>
+    <t>A. femoralis</t>
+  </si>
+  <si>
+    <t>artery; femoralis; femoral artery; thigh; atardamar</t>
+  </si>
+  <si>
+    <t>A. femoralis, uyluk bölgesini besleyen büyük bir arterdir.</t>
+  </si>
+  <si>
+    <t>["A. iliaca externa uyluk bölgesine ulaştığında a. femoralis adını alır.","Bu arter uyluk kaslarına dallar vererek bölgenin kanlanmasını sağlar.","Uyluk boyunca aşağı doğru ilerleyerek diz bölgesine ulaşır."]</t>
+  </si>
+  <si>
+    <t>poplitea</t>
+  </si>
+  <si>
+    <t>A. poplitea</t>
+  </si>
+  <si>
+    <t>artery; poplitea; popliteal artery; knee; atardamar</t>
+  </si>
+  <si>
+    <t>A. poplitea, diz arkasında bulunan ve diz bölgesini besleyen arterdir.</t>
+  </si>
+  <si>
+    <t>["A. femoralis diz bölgesine ulaştığında a. poplitea adını alır.","Bu arter dizin arka kısmında yer alır.","Diz çevresindeki yapıların beslenmesini sağlar."]</t>
+  </si>
+  <si>
+    <t>tibialis_anterior</t>
+  </si>
+  <si>
+    <t>A. tibialis anterior</t>
+  </si>
+  <si>
+    <t>artery; tibialis anterior; anterior tibial artery; leg; atardamar</t>
+  </si>
+  <si>
+    <t>A. tibialis anterior, bacağın ön kısmını besleyen arterdir.</t>
+  </si>
+  <si>
+    <t>["A. poplitea baldır bölgesinde iki ana dala ayrılır.","Bu dallardan biri a. tibialis anteriordur.","Bacağın ön kısmındaki kasların ve dokuların beslenmesini sağlar.","Ayak sırtında a. dorsalis pedis olarak devam eder."]</t>
+  </si>
+  <si>
+    <t>tibialis_posterior</t>
+  </si>
+  <si>
+    <t>A. tibialis posterior</t>
+  </si>
+  <si>
+    <t>artery; tibialis posterior; posterior tibial artery; leg; atardamar</t>
+  </si>
+  <si>
+    <t>A. tibialis posterior, bacağın arka bölümünü besleyen arterdir.</t>
+  </si>
+  <si>
+    <t>["A. poplitea baldır bölgesinde a. tibialis anterior ve a. tibialis posterior olarak ikiye ayrılır.","A. tibialis posterior bacağın arka bölümündeki kasları besler.","Alt bacak ve ayak bölgesinin kanlanmasına katkı sağlar."]</t>
+  </si>
+  <si>
+    <t>dorsalis_pedis</t>
+  </si>
+  <si>
+    <t>A. dorsalis pedis</t>
+  </si>
+  <si>
+    <t>artery; dorsalis pedis; foot artery; pulse; atardamar</t>
+  </si>
+  <si>
+    <t>A. dorsalis pedis, ayağın üst kısmında bulunan arterdir.</t>
+  </si>
+  <si>
+    <t>["A. tibialis anterior ayak sırtına ulaştığında a. dorsalis pedis adını alır.","Ayağın üst kısmındaki dokuların beslenmesini sağlar.","Birinci metatarsal aralıkta bu arter üzerinden nabız alınabilir."]</t>
+  </si>
+  <si>
+    <t>temporalis</t>
+  </si>
+  <si>
+    <t>A. temporalis</t>
+  </si>
+  <si>
+    <t>Head_Face</t>
+  </si>
+  <si>
+    <t>artery; temporalis; temporal artery; nabız; atardamar</t>
+  </si>
+  <si>
+    <t>A. temporalis, baş bölgesinde nabız alınabilen arterlerden biridir.</t>
+  </si>
+  <si>
+    <t>["Bu arter şakak bölgesinde bulunur.","Baş bölgesinde nabız değerlendirilirken bu damardan yararlanılabilir."]</t>
+  </si>
+  <si>
+    <t>Ders kitabı s.143</t>
+  </si>
+  <si>
+    <t>carotis_communis</t>
+  </si>
+  <si>
+    <t>A. carotis communis</t>
+  </si>
+  <si>
+    <t>Neck</t>
+  </si>
+  <si>
+    <t>artery; carotis communis; carotid artery; nabız; atardamar</t>
+  </si>
+  <si>
+    <t>A. carotis communis, boyun bölgesinde nabız alınabilen önemli arterlerden biridir.</t>
+  </si>
+  <si>
+    <t>["Bu arter boyunda yer alır.","Fiziksel muayenede karotis arterden nabız alınabilir.","Karotis arterden nabız alınırken dikkat edilmelidir."]</t>
+  </si>
+  <si>
+    <t>axillaris_pulse</t>
+  </si>
+  <si>
+    <t>artery; axillaris; axillary artery; nabız; atardamar</t>
+  </si>
+  <si>
+    <t>A. axillaris, üst ekstremitede nabız alınabilen arterlerden biridir.</t>
+  </si>
+  <si>
+    <t>["Bu arter koltuk altı bölgesinde bulunur.","Üst ekstremite arterlerinden biri olarak nabız değerlendirmesinde kullanılabilir."]</t>
+  </si>
+  <si>
+    <t>brachialis_pulse</t>
+  </si>
+  <si>
+    <t>artery; brachialis; brachial artery; nabız; atardamar</t>
+  </si>
+  <si>
+    <t>A. brachialis, üst ekstremitede nabız alınabilen arterlerden biridir.</t>
+  </si>
+  <si>
+    <t>["Bu arter kol bölgesinde bulunur.","Fiziksel muayenede üst ekstremite arterlerinden biri olarak nabız değerlendirilmesinde kullanılabilir."]</t>
+  </si>
+  <si>
+    <t>ulnaris_pulse</t>
+  </si>
+  <si>
+    <t>artery; ulnaris; ulnar artery; nabız; atardamar</t>
+  </si>
+  <si>
+    <t>A. ulnaris, ön kol bölgesinde bulunan arterlerden biridir.</t>
+  </si>
+  <si>
+    <t>["Bu arter ön kol bölgesinde yer alır.","Üst ekstremitede nabız alınabilen arterlerden biridir."]</t>
+  </si>
+  <si>
+    <t>radialis_pulse</t>
+  </si>
+  <si>
+    <t>artery; radialis; radial artery; nabız; atardamar</t>
+  </si>
+  <si>
+    <t>A. radialis, el bileğinde nabız alınmasında yaygın olarak kullanılan arterdir.</t>
+  </si>
+  <si>
+    <t>["Bu arter el bileği bölgesinde bulunur.","Rutin muayenelerde nabız genellikle radial arter üzerinden değerlendirilir."]</t>
+  </si>
+  <si>
+    <t>femoralis_pulse</t>
+  </si>
+  <si>
+    <t>artery; femoralis; femoral artery; nabız; atardamar</t>
+  </si>
+  <si>
+    <t>A. femoralis, alt ekstremitede nabız alınabilen arterlerden biridir.</t>
+  </si>
+  <si>
+    <t>["Bu arter uyluk bölgesinde bulunur.","Alt ekstremite arterlerinden biri olarak nabız değerlendirilmesinde kullanılabilir."]</t>
+  </si>
+  <si>
+    <t>poplitea_pulse</t>
+  </si>
+  <si>
+    <t>artery; poplitea; popliteal artery; nabız; atardamar</t>
+  </si>
+  <si>
+    <t>A. poplitea, diz arkasında bulunan arterdir.</t>
+  </si>
+  <si>
+    <t>["Bu arter dizin arka kısmında yer alır.","Alt ekstremitede nabız değerlendirilirken bu damardan yararlanılabilir."]</t>
+  </si>
+  <si>
+    <t>tibialis_posterior_pulse</t>
+  </si>
+  <si>
+    <t>artery; tibialis posterior; posterior tibial artery; nabız; atardamar</t>
+  </si>
+  <si>
+    <t>A. tibialis posterior, alt bacak bölgesinde nabız alınabilen arterlerden biridir.</t>
+  </si>
+  <si>
+    <t>["Bu arter baldır bölgesinde yer alır.","Alt ekstremitede nabız değerlendirilmesinde kullanılan arterlerden biridir."]</t>
+  </si>
+  <si>
+    <t>dorsalis_pedis_pulse</t>
+  </si>
+  <si>
+    <t>Foot</t>
+  </si>
+  <si>
+    <t>artery; dorsalis pedis; foot artery; nabız; atardamar</t>
+  </si>
+  <si>
+    <t>["Bu arter ayak sırtında bulunur.","Alt ekstremitede nabız değerlendirilirken bu damardan yararlanılabilir."]</t>
+  </si>
+  <si>
+    <t>veins</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Venae  </t>
+  </si>
+  <si>
+    <t>vein; vena; ven; circulation; toplardamar</t>
+  </si>
+  <si>
+    <t>Toplardamarlar, kanı dokular ve akciğerlerden kalbe taşıyan damar grubudur.</t>
+  </si>
+  <si>
+    <t>["Temiz kanı akciğerlerden kalbe taşıyan akciğer toplardamarları dışında venler kirli kan taşır.","Venlerde kan basıncı arterlere göre daha düşüktür.","Ven duvarları arterlere göre daha incedir.","Normal istirahat halinde dolaşımdaki kanın büyük bir bölümü venlerde bulunur."]</t>
+  </si>
+  <si>
+    <t>Ders kitabı s.140</t>
+  </si>
+  <si>
+    <t>upper_extremity_veins</t>
+  </si>
+  <si>
+    <t>Üst ekstremite venleri</t>
+  </si>
+  <si>
+    <t>vein; upper extremity veins; arm veins; vena; toplardamar</t>
+  </si>
+  <si>
+    <t>Üst ekstremite venleri, kol bölgesindeki kirli kanı kalbe doğru taşıyan toplardamarlardır.</t>
+  </si>
+  <si>
+    <t>["Üst ekstremite venleri yüzeysel ve derin venler olmak üzere iki grupta incelenir.","Yüzeysel venler deri altında seyreder ve görülebilir.","Önemli yüzeysel venler arasında v. cephalica, v. basilica, v. mediana antebrachii ve v. mediana cubiti bulunur.","Derin venler arterlerle birlikte seyreder.","Önemli derin venler arasında v. radialis, v. ulnaris, v. brachialis ve v. axillaris yer alır.","Üst ekstremiteden gelen venöz kan v. subclavia üzerinden daha büyük venlere taşınır."]</t>
+  </si>
+  <si>
+    <t>brachiocephalica_vein</t>
+  </si>
+  <si>
+    <t>V. brachiocephalica</t>
+  </si>
+  <si>
+    <t>vein; brachiocephalica; brachiocephalic vein; toplardamar</t>
+  </si>
+  <si>
+    <t>V. brachiocephalica, kol ve baş bölgesinden gelen venlerin birleşmesi ile oluşur.</t>
+  </si>
+  <si>
+    <t>["Baş bölgesinden gelen v. jugularis interna ile boynun dış venlerinden v. jugularis externa birleşir.","Koldan gelen v. subclavia ile birleşerek v. brachiocephalica oluşur."]</t>
+  </si>
+  <si>
+    <t>jugularis_interna</t>
+  </si>
+  <si>
+    <t>V. jugularis interna</t>
+  </si>
+  <si>
+    <t>vein; jugularis interna; internal jugular vein; toplardamar</t>
+  </si>
+  <si>
+    <t>V. jugularis interna boyundaki en büyük vendir.</t>
+  </si>
+  <si>
+    <t>["El sırtının ulnar tarafından başlar.","Ön kolun iç yüzünden yukarı doğru ilerler.","Dirsek bölgesini geçerek kol bölgesine ulaşır.","Kol bölgesinde derine ilerler ve derin venöz sistemle birleşerek v. axillaris'in oluşumuna katılır."]</t>
+  </si>
+  <si>
+    <t>jugularis_externa</t>
+  </si>
+  <si>
+    <t>V. jugularis externa</t>
+  </si>
+  <si>
+    <t>vein; jugularis externa; external jugular vein; toplardamar</t>
+  </si>
+  <si>
+    <t>V. jugularis externa başın dış venlerini ve yüzün yüzeysel venlerini toplar.</t>
+  </si>
+  <si>
+    <t>["Baş ve yüzün yüzeysel venleri ile birleşir.","Boyundan aşağı doğru ilerler.","V. subclavia ile birleşerek sonlanır."]</t>
+  </si>
+  <si>
+    <t>subclavia_vein</t>
+  </si>
+  <si>
+    <t>V. subclavia</t>
+  </si>
+  <si>
+    <t>vein; subclavia; subclavian vein; toplardamar</t>
+  </si>
+  <si>
+    <t>V. subclavia, v. axillaris'in köprücük kemiği altındaki devamı olan vendir.</t>
+  </si>
+  <si>
+    <t>["Kol venleri birleşerek v. axillaris'i oluşturur.","V. axillaris köprücük kemiğinin altında v. subclavia adını alır.","Buradan jugular venlerle birleşerek v. brachiocephalica'yı oluşturur."]</t>
+  </si>
+  <si>
+    <t>axillaris_vein</t>
+  </si>
+  <si>
+    <t>V. axillaris</t>
+  </si>
+  <si>
+    <t>vein; axillaris; axillary vein; toplardamar</t>
+  </si>
+  <si>
+    <t>V. axillaris, üst ekstremitenin derin venöz dönüşünde yer alan ve koltuk altı bölgesinde bulunan büyük bir vendir.</t>
+  </si>
+  <si>
+    <t>["Kol bölgesindeki venlerin birleşmesi ile oluşur.","Koltuk altı bölgesinde bulunur.","Yukarı doğru ilerleyerek v. subclavia olarak devam eder."]</t>
+  </si>
+  <si>
+    <t>cephalica_vein</t>
+  </si>
+  <si>
+    <t>V. cephalica</t>
+  </si>
+  <si>
+    <t>vein; cephalica; cephalic vein; toplardamar</t>
+  </si>
+  <si>
+    <t>V. cephalica üst ekstremitenin önemli yüzeysel venlerinden biridir.</t>
+  </si>
+  <si>
+    <t>["El sırtının radyal tarafından başlar.","Ön kolun ön tarafına doğru ilerler.","Kolun dış yanından yukarı çıkar.","Proksimalde v. axillaris'e katılır."]</t>
+  </si>
+  <si>
+    <t>brachialis_vein</t>
+  </si>
+  <si>
+    <t>V. brachialis</t>
+  </si>
+  <si>
+    <t>vein; brachialis; brachial vein; toplardamar</t>
+  </si>
+  <si>
+    <t>V. brachialis kol bölgesinin derin venlerinden biridir.</t>
+  </si>
+  <si>
+    <t>["V. radialis ve v. ulnaris'in dirsek önünde birleşmesi ile oluşur.","Yukarı doğru ilerleyerek v. axillaris'e katılır."]</t>
+  </si>
+  <si>
+    <t>basilica_vein</t>
+  </si>
+  <si>
+    <t>V. basilica</t>
+  </si>
+  <si>
+    <t>vein; basilica; basilic vein; toplardamar</t>
+  </si>
+  <si>
+    <t>V. basilica üst ekstremitenin önemli yüzeysel venlerinden biridir.</t>
+  </si>
+  <si>
+    <t>mediana_cubiti</t>
+  </si>
+  <si>
+    <t>V. mediana cubiti</t>
+  </si>
+  <si>
+    <t>vein; mediana cubiti; median cubital vein; toplardamar</t>
+  </si>
+  <si>
+    <t>V. mediana cubiti dirsek bölgesinde bulunan yüzeysel vendir.</t>
+  </si>
+  <si>
+    <t>["Dirsek ekleminin iç yüzünde bulunur.","V. basilica ile v. cephalica'yı birbirine bağlar."]</t>
+  </si>
+  <si>
+    <t>antebrachii_mediana</t>
+  </si>
+  <si>
+    <t>V. antebrachii mediana</t>
+  </si>
+  <si>
+    <t>vein; antebrachii mediana; median antebrachial vein; toplardamar</t>
+  </si>
+  <si>
+    <t>V. antebrachii mediana ön kolun yüzeysel venlerinden biridir.</t>
+  </si>
+  <si>
+    <t>["Elin palmar yüzünden başlayarak yukarı doğru uzanır.","V. mediana cubiti veya v. basilica ile birleşir."]</t>
+  </si>
+  <si>
+    <t>radialis_vein</t>
+  </si>
+  <si>
+    <t>V. radialis</t>
+  </si>
+  <si>
+    <t>vein; radialis; radial vein; toplardamar</t>
+  </si>
+  <si>
+    <t>V. radialis el ve ön kolun radyal bölgesinin venöz kanını toplar.</t>
+  </si>
+  <si>
+    <t>["El ve ön kolun radyal tarafındaki kirli kanı toplar.","V. ulnaris ile birleşerek v. brachialisi oluşturur."]</t>
+  </si>
+  <si>
+    <t>ulnaris_vein</t>
+  </si>
+  <si>
+    <t>V. ulnaris</t>
+  </si>
+  <si>
+    <t>vein; ulnaris; ulnar vein; toplardamar</t>
+  </si>
+  <si>
+    <t>V. ulnaris el ve ön kolun ulnar bölgesinin venöz kanını toplar.</t>
+  </si>
+  <si>
+    <t>["El ve ön kolun ulnar tarafındaki kirli kanı toplar.","V. radialis ile birleşerek v. brachialisi oluşturur."]</t>
+  </si>
+  <si>
+    <t>cava_superior</t>
+  </si>
+  <si>
+    <t>V. cava superior</t>
+  </si>
+  <si>
+    <t>Thorax</t>
+  </si>
+  <si>
+    <t>vein; cava superior; superior vena cava; toplardamar</t>
+  </si>
+  <si>
+    <t>V. cava superior, baş, boyun, göğüs ve üst ekstremite bölgelerinden gelen venöz kanı kalbe taşıyan büyük bir toplardamardır.</t>
+  </si>
+  <si>
+    <t>["V. cava superior iki adet v. brachiocephalicanın birleşmesi ile oluşur.","Baş, boyun, göğüs ve üst ekstremite bölgelerinden gelen kirli kanı toplar.","Topladığı kanı kalbin sağ atriumuna taşır."]</t>
+  </si>
+  <si>
+    <t>lower_extremity_veins</t>
+  </si>
+  <si>
+    <t>Alt ekstremite venleri</t>
+  </si>
+  <si>
+    <t>vein; lower extremity veins; leg veins; vena; toplardamar</t>
+  </si>
+  <si>
+    <t>Alt ekstremite venleri bacak ve ayak bölgesindeki venöz kanı kalbe doğru taşıyan toplardamarlardır.</t>
+  </si>
+  <si>
+    <t>["Alt ekstremite venleri yüzeysel ve derin venler olmak üzere iki grupta incelenir.","Yüzeysel venlerin yapısında kapakçıklar bulunur.","Derin venler genellikle aynı isimdeki arterlerle birlikte seyreder.","Alt ekstremiteden gelen venöz kan daha büyük venler aracılığıyla v. cava inferiora taşınır."]</t>
+  </si>
+  <si>
+    <t>Ders kitabı s.141</t>
+  </si>
+  <si>
+    <t>cava_inferior</t>
+  </si>
+  <si>
+    <t>V. cava inferior</t>
+  </si>
+  <si>
+    <t>vein; cava inferior; inferior vena cava; toplardamar</t>
+  </si>
+  <si>
+    <t>V. cava inferior gövdenin alt bölümünden gelen venöz kanı kalbe taşıyan büyük bir vendir.</t>
+  </si>
+  <si>
+    <t>["Gövdede diyaframın altında kalan bölüm ile alt ekstremite bölgelerinin kanını toplar.","Sağ ve sol v. iliaca communis'in birleşmesi ile oluşur.","Topladığı kanı kalbin sağ atriumuna taşır."]</t>
+  </si>
+  <si>
+    <t>iliaca_communis_vein</t>
+  </si>
+  <si>
+    <t>V. iliaca communis</t>
+  </si>
+  <si>
+    <t>Pelvis</t>
+  </si>
+  <si>
+    <t>vein; iliaca communis; common iliac vein; toplardamar</t>
+  </si>
+  <si>
+    <t>V. iliaca communis pelvis ve alt ekstremitenin venöz kanını taşıyan vendir.</t>
+  </si>
+  <si>
+    <t>["V. iliaca interna ve v. iliaca externa venlerinin birleşmesi ile oluşur.","Sağ ve sol v. iliaca communis venleri birleşerek v. cava inferioru oluşturur."]</t>
+  </si>
+  <si>
+    <t>iliaca_externa_vein</t>
+  </si>
+  <si>
+    <t>V. iliaca externa</t>
+  </si>
+  <si>
+    <t>vein; iliaca externa; external iliac vein; toplardamar</t>
+  </si>
+  <si>
+    <t>V. iliaca externa alt ekstremitenin venöz kanını taşıyan önemli venlerden biridir.</t>
+  </si>
+  <si>
+    <t>["Alt ekstremiteden gelen venöz kanı taşır.","Kasık bölgesinden aşağıda v. femoralis adını alır."]</t>
+  </si>
+  <si>
+    <t>femoralis_vein</t>
+  </si>
+  <si>
+    <t>V. femoralis</t>
+  </si>
+  <si>
+    <t>vein; femoralis; femoral vein; toplardamar</t>
+  </si>
+  <si>
+    <t>V. femoralis bacak bölgesinin venöz kanını taşıyan önemli derin vendir.</t>
+  </si>
+  <si>
+    <t>["Bacak bölgesinin kirli kanını taşır.","V. popliteanın devamıdır.","Yukarı doğru ilerleyerek kasık bölgesinde v. iliaca externa adını alır."]</t>
+  </si>
+  <si>
+    <t>poplitea_vein</t>
+  </si>
+  <si>
+    <t>V. poplitea</t>
+  </si>
+  <si>
+    <t>vein; poplitea; popliteal vein; toplardamar</t>
+  </si>
+  <si>
+    <t>V. poplitea diz arkasında bulunan derin vendir.</t>
+  </si>
+  <si>
+    <t>["V. tibialis anterior ve v. tibialis posteriorun birleşmesi ile oluşur.","Diz arkasından yukarı doğru ilerler.","Yukarıda v. femoralis adını alır."]</t>
+  </si>
+  <si>
+    <t>tibialis_anterior_vein</t>
+  </si>
+  <si>
+    <t>V. tibialis anterior</t>
+  </si>
+  <si>
+    <t>vein; tibialis anterior; anterior tibial vein; toplardamar</t>
+  </si>
+  <si>
+    <t>V. tibialis anterior ayak ve bacağın ön bölümünden gelen venöz kanı taşır.</t>
+  </si>
+  <si>
+    <t>["Ayak sırtından başlayarak baldırın önünden yukarı doğru ilerler.","V. tibialis posterior ile birleşerek v. popliteayı oluşturur."]</t>
+  </si>
+  <si>
+    <t>tibialis_posterior_vein</t>
+  </si>
+  <si>
+    <t>V. tibialis posterior</t>
+  </si>
+  <si>
+    <t>vein; tibialis posterior; posterior tibial vein; toplardamar</t>
+  </si>
+  <si>
+    <t>V. tibialis posterior ayak tabanı ve baldır bölgesinin venöz kanını taşır.</t>
+  </si>
+  <si>
+    <t>["Ayak tabanından başlayarak baldırın arka kısmından yukarı doğru ilerler.","V. tibialis anterior ile birleşerek v. popliteayı oluşturur."]</t>
+  </si>
+  <si>
+    <t>saphena_magna</t>
+  </si>
+  <si>
+    <t>V. saphena magna</t>
+  </si>
+  <si>
+    <t>vein; saphena magna; great saphenous vein; toplardamar</t>
+  </si>
+  <si>
+    <t>V. saphena magna vücudun en uzun venidir.</t>
+  </si>
+  <si>
+    <t>["Ayak sırtından başlar.","Bacağın iç yüzünden yukarı doğru ilerler.","Kasık bölgesinde v. femoralis ile birleşir.","Koroner arter bypass ameliyatlarında greft olarak kullanılabilir."]</t>
+  </si>
+  <si>
+    <t>saphena_parva</t>
+  </si>
+  <si>
+    <t>V. saphena parva</t>
+  </si>
+  <si>
+    <t>vein; saphena parva; small saphenous vein; toplardamar</t>
+  </si>
+  <si>
+    <t>V. saphena parva alt ekstremitenin yüzeysel venlerinden biridir.</t>
+  </si>
+  <si>
+    <t>["Ayak sırtının dış tarafından başlar.","Baldırın arka kısmından yukarı doğru ilerler.","Diz arkasında derine ilerleyerek v. popliteaya bağlanır."]</t>
+  </si>
+  <si>
+    <t>systemic_circulation</t>
+  </si>
+  <si>
+    <t>Büyük kan dolaşımı</t>
+  </si>
+  <si>
+    <t>Circulation</t>
+  </si>
+  <si>
+    <t>circulation; systemic; large_circulation; heart; body</t>
+  </si>
+  <si>
+    <t>Büyük kan dolaşımı, oksijen bakımından zengin kanın kalpten çıkarak tüm vücut dokularına gönderilmesini ve dokularda oluşan karbondioksit ile atık maddelerin toplanarak tekrar kalbe getirilmesini sağlayan dolaşımdır.</t>
+  </si>
+  <si>
+    <t>["Oksijenlenmiş kan pulmoner venler ile sol atriyuma gelir", "Kan mitral kapaktan geçerek sol ventriküle ulaşır", "Sol ventrikül kasılarak kanı aort aracılığıyla tüm vücuda pompalar", "Dokularda gaz değişimi gerçekleşir ve kan kirlenir", "Kirli kan vena cava ile sağ atriyuma geri döner"]</t>
+  </si>
+  <si>
+    <t>Ders kitabı s.145</t>
+  </si>
+  <si>
+    <t>pulmonary_circulation</t>
+  </si>
+  <si>
+    <t>Küçük kan dolaşımı</t>
+  </si>
+  <si>
+    <t>circulation; pulmonary; small_circulation; heart; lung</t>
+  </si>
+  <si>
+    <t>Küçük kan dolaşımı, kalpten akciğerlere gönderilen kirli kanın akciğerlerde oksijenlenerek temizlenmesi ve tekrar kalbe dönmesini sağlayan dolaşımdır.</t>
+  </si>
+  <si>
+    <t>["Kirli kan sağ atriyuma gelir", "Kan triküspit kapaktan geçerek sağ ventriküle ulaşır", "Sağ ventrikül kasılarak kanı pulmoner arter aracılığıyla akciğerlere pompalar", "Akciğerlerde gaz değişimi gerçekleşir ve kan oksijenlenir", "Oksijenlenmiş kan pulmoner venler ile sol atriyuma geri döner"]</t>
+  </si>
+  <si>
+    <t>systemic_left_ventricle_01</t>
+  </si>
+  <si>
+    <t>Sol ventrikül</t>
+  </si>
+  <si>
+    <t>circulation; systemic; large_circulation; heart; ventricle</t>
+  </si>
+  <si>
+    <t>Sol ventrikül, oksijen bakımından zengin kanı aort aracılığıyla tüm vücuda pompalayan ve büyük kan dolaşımının başladığı kalp odacığıdır.</t>
+  </si>
+  <si>
+    <t>["Sol atriyumdan gelen oksijenli kan sol ventrikülde toplanır", "Ventrikül kasılarak kanı kalpten dışarı pompalar", "Kan aort damarına gönderilir"]</t>
+  </si>
+  <si>
+    <t>systemic_aorta_02</t>
+  </si>
+  <si>
     <t>Aort</t>
   </si>
   <si>
-    <t>heart; vessel; artery; aorta</t>
-  </si>
-  <si>
-    <t>Aort, kalpten çıkan en büyük atardamardır.</t>
-  </si>
-  <si>
-    <t>["Sol karıncıktan çıkan oksijen bakımından zengin kanı tüm vücuda taşır." , "Aort, sistemik dolaşımın başlangıç damarıdır."]</t>
-  </si>
-  <si>
-    <t>pulmonary_vein</t>
-  </si>
-  <si>
-    <t>Akciğer toplardamarı</t>
-  </si>
-  <si>
-    <t>heart; vessel; vein; pulmonary</t>
-  </si>
-  <si>
-    <t>Akciğer toplardamarı, akciğerlerde oksijenlenen kanı kalbin sol kulakçığına taşıyan damardır.</t>
-  </si>
-  <si>
-    <t>["Akciğerlerden gelen oksijen bakımından zengin kanı kalbe getirir.", "Diğer toplardamarlardan farklı olarak oksijen bakımından zengin kan taşır."]</t>
-  </si>
-  <si>
-    <t>heart_valves</t>
-  </si>
-  <si>
-    <t>Kalbin kapakları</t>
-  </si>
-  <si>
-    <t>heart; valve; mitral; tricuspid; aortic; pulmonary</t>
-  </si>
-  <si>
-    <t>Kalpte dört adet kapak bulunur.</t>
-  </si>
-  <si>
-    <t>["Bu kapakların ikisi atriyoventriküler kapaklar, ikisi ise semilunar kapaklardır." , "Atriyoventriküler kapaklar, kulakçıklar ile karıncıklar arasında yer alır ve mitral kapak ile triküspit kapaktan oluşur." , "Semilunar kapaklar ise karıncıklar ile büyük atardamarlar arasında bulunur ve aort kapağı ile pulmoner kapaktan oluşur.", "Kalp kapakları, kalbin kasılması ve gevşemesi sırasında kanın geriye doğru akmasını engelleyerek kanın tek yönlü ilerlemesini sağlar."]</t>
-  </si>
-  <si>
-    <t>Ders kitabı s.132</t>
-  </si>
-  <si>
-    <t>coronary_arteries</t>
-  </si>
-  <si>
-    <t>Koroner arterler</t>
-  </si>
-  <si>
-    <t>heart; coronary; artery; circulation</t>
-  </si>
-  <si>
-    <t>Kalp kasına oksijen bakımından zengin kan taşıyan damarlara koroner arterler denir.</t>
-  </si>
-  <si>
-    <t>["Koroner arterler aorttan ayrılan ilk dallardır." , "Sağ koroner arter kalbin sağ tarafını, sol koroner arter ise kalbin sol tarafını besler." , "Bu damarlarda oluşan daralma veya tıkanıklıklar kalp kasının yeterince beslenmesini engelleyebilir ve kalp krizine neden olabilir."]</t>
-  </si>
-  <si>
-    <t>arteria_coronalis_dextra</t>
-  </si>
-  <si>
-    <t>Arteria coronalis dextra</t>
-  </si>
-  <si>
-    <t>heart; coronary; artery; right</t>
-  </si>
-  <si>
-    <t>Sağ koroner arter (arteria coronalis dextra), aorttan ayrılan ve kalbin sağ tarafını besleyen koroner damardır.</t>
-  </si>
-  <si>
-    <t>["Aorttan ayrılan ilk dallardan biridir.", "Kalp kasına oksijen ve besin bakımından zengin kan taşır."]</t>
-  </si>
-  <si>
-    <t>arteria_coronalis_sinistra</t>
-  </si>
-  <si>
-    <t>Arteria coronalis sinistra</t>
-  </si>
-  <si>
-    <t>heart; coronary; artery; left</t>
-  </si>
-  <si>
-    <t>Sol koroner arter (arteria coronalis sinistra), aorttan ayrılan ve kalbin sol tarafını besleyen koroner damardır.</t>
-  </si>
-  <si>
-    <t>["Kalp kasının büyük bölümüne oksijen bakımından zengin kan taşır."]</t>
-  </si>
-  <si>
-    <t>vena_cordis_magna</t>
-  </si>
-  <si>
-    <t>Vena cordis magna</t>
-  </si>
-  <si>
-    <t>heart; coronary; vein</t>
-  </si>
-  <si>
-    <t>Vena cordis magna, kalp kasından toplanan kirli kanı taşıyan büyük koroner toplardamarlardan biridir.</t>
-  </si>
-  <si>
-    <t>["Bu damar kalbin yüzeyindeki venlerle birleşerek koroner sinüse katılır."]</t>
-  </si>
-  <si>
-    <t>vena_cordis_media</t>
-  </si>
-  <si>
-    <t>Vena cordis media</t>
-  </si>
-  <si>
-    <t>Vena cordis media, kalp kasından gelen kirli kanı toplayan koroner toplardamarlardan biridir.</t>
-  </si>
-  <si>
-    <t>["Bu damar da diğer koroner venlerle birlikte koroner sinüse açılır."]</t>
-  </si>
-  <si>
-    <t>vena_cordis_parva</t>
-  </si>
-  <si>
-    <t>Vena cordis parva</t>
-  </si>
-  <si>
-    <t>Vena cordis parva, kalp kasından gelen kirli kanı taşıyan küçük koroner toplardamarlardan biridir.</t>
-  </si>
-  <si>
-    <t>["Bu damar koroner venlerle birleşerek koroner sinüse katılır."]</t>
-  </si>
-  <si>
-    <t>coronary_sinus</t>
-  </si>
-  <si>
-    <t>Sinus coronarius</t>
-  </si>
-  <si>
-    <t>heart; coronary; sinus</t>
-  </si>
-  <si>
-    <t>Sinus coronarius, kalp kasından gelen kirli kanın toplandığı geniş bir toplardamardır.</t>
-  </si>
-  <si>
-    <t>["Koroner venler burada birleşir ve kan buradan sağ atriyuma dökülür."]</t>
-  </si>
-  <si>
-    <t>cardiac_cycle</t>
-  </si>
-  <si>
-    <t>Kalbin çalışması</t>
-  </si>
-  <si>
-    <t>heart; cardiac cycle; systole; diastole</t>
-  </si>
-  <si>
-    <t>Kalp, kendine ait uyarı çıkaran hücreler sayesinde düzenli olarak kasılıp gevşer.</t>
-  </si>
-  <si>
-    <t>["Kalbin kasılma evresine sistol, gevşeme evresine ise diyastol denir." , "Ventriküller kasıldığında kan atardamarlara pompalanır, gevşediğinde ise atriyumlardan gelen kan ventriküllere dolar." , "Kapaklar kanın tek yönlü ilerlemesini sağlar ve geri kaçmasını engeller."]</t>
-  </si>
-  <si>
-    <t>Ders kitabı s.134</t>
-  </si>
-  <si>
-    <t>tricuspid_valve</t>
-  </si>
-  <si>
-    <t>Triküspit kapak</t>
-  </si>
-  <si>
-    <t>heart; valve; tricuspid</t>
-  </si>
-  <si>
-    <t>Triküspit kapak, sağ kulakçık ile sağ karıncık arasında bulunan atriyoventriküler kapaktır.</t>
-  </si>
-  <si>
-    <t>["Ventrikül kasıldığında kanın tekrar kulakçığa geri dönmesini engeller."]</t>
-  </si>
-  <si>
-    <t>mitral_valve</t>
-  </si>
-  <si>
-    <t>Mitral kapak</t>
-  </si>
-  <si>
-    <t>heart; valve; mitral</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mitral kapak, sol kulakçık ile sol karıncık arasında bulunan atriyoventriküler kapaktır. </t>
-  </si>
-  <si>
-    <t>["Kanın ventrikül kasılması sırasında sol kulakçığa geri kaçmasını engeller."]</t>
-  </si>
-  <si>
-    <t>myocardium</t>
-  </si>
-  <si>
-    <t>Myocardium</t>
-  </si>
-  <si>
-    <t>heart; muscle; myocardium</t>
-  </si>
-  <si>
-    <t>Myokard, kalbin kasılmasını sağlayan kalın kas tabakasıdır.</t>
-  </si>
-  <si>
-    <t>["Bu kas tabakası kasılarak kanın kalpten damarlara pompalanmasını sağlar."]</t>
-  </si>
-  <si>
-    <t>arteries</t>
-  </si>
-  <si>
-    <t>Atardamarlar</t>
-  </si>
-  <si>
-    <t>Vessels</t>
-  </si>
-  <si>
-    <t>artery; arter; vessel; blood circulation; damar</t>
-  </si>
-  <si>
-    <t>Atardamarlar, kanı kalpten dokulara ve organlara taşıyan kan damarlarıdır.</t>
-  </si>
-  <si>
-    <t>["Atardamarlar kalbin ventrikülleri ile bağlantılı damarlardır ve kanı kalpten uzaklaştırarak vücudun farklı bölgelerine taşırlar.", "Sağ ventrikülden akciğerlere kirli kan taşıyan akciğer atardamarı dışında diğer tüm atardamarlar oksijen bakımından zengin temiz kan taşır.", "Sol ventrikülden çıkan temiz kan sistol sırasında aort damarına pompalanır ve buradan vücuttaki diğer atardamarlara dağıtılır.", "Atardamarların çapları perifer bölgelere doğru gidildikçe küçülür ve bu küçük damarlara arteriyol adı verilir.", "Atardamarlarda kan basıncı yüksek olduğu için damar duvarları toplardamarlara göre daha kalın ve dayanıklıdır."]</t>
-  </si>
-  <si>
-    <t>Ders kitabı s.138</t>
-  </si>
-  <si>
-    <t>upper_extremity_arteries</t>
-  </si>
-  <si>
-    <t>Üst ekstremite arterleri</t>
-  </si>
-  <si>
-    <t>Upper_Extremity</t>
-  </si>
-  <si>
-    <t>artery; arter; upper extremity; arm; kol; damar; subclavian; axillary; brachial; radial; ulnar</t>
-  </si>
-  <si>
-    <t>Üst ekstremite arterleri, omuzdan ele kadar üst ekstremiteyi besleyen atardamarlardır.</t>
-  </si>
-  <si>
-    <t>["Sağ ve sol köprücük altı arterleri kola doğru ilerledikçe çapları giderek küçülür ve geçtikleri bölgeye göre farklı isimler alırlar.","Üst ekstremitede arterler sırasıyla a. subclavia, a. axillaris, a. brachialis, a. radialis ve a. ulnaris olarak devam eder.","Bu damarlar omuz, kol, ön kol ve elin kanlanmasını sağlar."]</t>
-  </si>
-  <si>
-    <t>subclavian_artery</t>
-  </si>
-  <si>
-    <t>A. subclavia</t>
-  </si>
-  <si>
-    <t>artery; subclavian artery; a. subclavia; upper extremity; arter; köprücük altı atardamarı; atardamar</t>
-  </si>
-  <si>
-    <t>A. subclavia, üst ekstremiteye kan taşıyan ana arterlerden biridir.</t>
-  </si>
-  <si>
-    <t>["Sağ ve sol a. subclavia, üst ekstremiteye uzanan arteriyel dolaşımın başlangıç bölümünü oluşturur.","Bu damar kola doğru ilerledikçe bulunduğu bölgeye göre isim değiştirir.","Koltuk altı bölgesine ulaştığında a. axillaris adını alır."]</t>
-  </si>
-  <si>
-    <t>axillary_artery</t>
-  </si>
-  <si>
-    <t>A. axillaris</t>
-  </si>
-  <si>
-    <t>artery; arter; axillary artery; a. axillaris; koltuk altı atardamarı; upper extremity; atardamar</t>
-  </si>
-  <si>
-    <t>A. axillaris, a. subclavia'nın koltuk altı bölgesindeki devamıdır.</t>
-  </si>
-  <si>
-    <t>["A. subclavia, koltuk altı bölgesine geldiğinde a. axillaris adını alır.","A. axillaris göğüs ve omuz bölgesine dallar verir.","Bu damar kol bölgesine doğru devam ederek a. brachialis adını alır."]</t>
-  </si>
-  <si>
-    <t>brachial_artery</t>
-  </si>
-  <si>
-    <t>A. brachialis</t>
-  </si>
-  <si>
-    <t>artery; arter; brachial artery; a. brachialis; kol atardamarı; blood pressure; atardamar</t>
-  </si>
-  <si>
-    <t>A. brachialis, a. axillaris'in kol bölgesindeki devamıdır.</t>
-  </si>
-  <si>
-    <t>["A. axillaris kol bölgesine geçince a. brachialis adını alır.","A. brachialis kol kaslarının beslenmesini sağlar.","Tansiyon ölçümü klinikte bu damar üzerinden yapılır.","Dirsek ön bölgesinde a. radialis ve a. ulnaris olmak üzere iki dala ayrılır."]</t>
-  </si>
-  <si>
-    <t>radial_artery</t>
-  </si>
-  <si>
-    <t>A. radialis</t>
-  </si>
-  <si>
-    <t>artery; arter; radial artery; a. radialis; radius; nabız; pulse; upper extremity; atardamar</t>
-  </si>
-  <si>
-    <t>A. radialis, a. brachialis'in dirsek ön bölgesinde ayrılan dallarından biridir.</t>
-  </si>
-  <si>
-    <t>["A. brachialis dirsek ön bölgesinde a. radialis ve a. ulnaris olarak iki dala ayrılır.","A. radialis ön kolun ve elin bir bölümünün kanlanmasına katkı sağlar.","A. radialis nabız almada daha sık tercih edilen damarlardan biridir."]</t>
-  </si>
-  <si>
-    <t>ulnar_artery</t>
-  </si>
-  <si>
-    <t>A. ulnaris</t>
-  </si>
-  <si>
-    <t>artery; arter; ulnar artery; a. ulnaris; ulna; upper extremity; atardamar</t>
-  </si>
-  <si>
-    <t>A. ulnaris, a. brachialis'in dirsek ön bölgesinde ayrılan dallarından biridir.</t>
-  </si>
-  <si>
-    <t>["A. brachialis dirsek ön bölgesinde iki ana dala ayrılır ve bunlardan biri a. ulnaris'tir.","A. ulnaris ön kolun ve elin bir bölümünün kanlanmasına katkı sağlar.","A. ulnaris, a. radialis ile birlikte el bileği ve elin beslenmesinde görev alır."]</t>
-  </si>
-  <si>
-    <t>abdominal_aorta</t>
-  </si>
-  <si>
-    <t>Karın aortu</t>
-  </si>
-  <si>
-    <t>Abdomen</t>
-  </si>
-  <si>
-    <t>artery; abdominal aorta; aorta abdominalis; circulation; abdomen; atardamar</t>
-  </si>
-  <si>
-    <t>Karın aortu, aortun diyaframdan sonra karın boşluğunda devam eden bölümüdür.</t>
-  </si>
-  <si>
-    <t>["Karın aortu diyaframdan başlayarak bel omurları boyunca aşağı doğru uzanır.","Bu damar karın bölgesindeki birçok organa kan taşıyan arterlerin çıktığı ana damardır.","Truncus coeliacus, a. mesenterica superior ve a. mesenterica inferior gibi önemli arterler karın aortundan ayrılır.","Karın aortu yaklaşık dördüncü bel omuru hizasında ikiye ayrılarak sağ ve sol a. iliaca communis arterlerini oluşturur."]</t>
-  </si>
-  <si>
-    <t>truncus_coeliacus</t>
-  </si>
-  <si>
-    <t>Truncus coeliacus</t>
-  </si>
-  <si>
-    <t>artery; truncus coeliacus; celiac trunk; abdominal aorta; atardamar</t>
-  </si>
-  <si>
-    <t>Truncus coeliacus, karın aortundan ayrılan ve üç ana dala ayrılan önemli bir arterdir.</t>
-  </si>
-  <si>
-    <t>["Truncus coeliacus karın aortundan ayrılır.","Bu damar üç ana dala ayrılarak karın bölgesindeki bazı organlara kan taşır.","Dalları mide, karaciğer ve dalak gibi organların beslenmesine katkı sağlar."]</t>
-  </si>
-  <si>
-    <t>gastrica_sinistra</t>
-  </si>
-  <si>
-    <t>A. gastrica sinistra</t>
-  </si>
-  <si>
-    <t>artery; gastrica sinistra; left gastric artery; stomach; atardamar</t>
-  </si>
-  <si>
-    <t>A. gastrica sinistra, mideyi besleyen arterlerden biridir.</t>
-  </si>
-  <si>
-    <t>["Bu damar karın aortundan çıkan truncus coeliacusun dallarından biridir.","Midenin üst kısmına kan taşır.","Mide duvarının beslenmesine katkı sağlar."]</t>
-  </si>
-  <si>
-    <t>hepatica_communis</t>
-  </si>
-  <si>
-    <t>A. hepatica communis</t>
-  </si>
-  <si>
-    <t>artery; hepatica communis; common hepatic artery; liver; atardamar</t>
-  </si>
-  <si>
-    <t>A. hepatica communis, karaciğeri besleyen önemli arterlerden biridir.</t>
-  </si>
-  <si>
-    <t>["Bu damar truncus coeliacusun ana dallarından biridir.","Karaciğere kan taşır.","Karaciğer dokusunun beslenmesinde görev alır."]</t>
-  </si>
-  <si>
-    <t>lienalis</t>
-  </si>
-  <si>
-    <t>A. lienalis</t>
-  </si>
-  <si>
-    <t>artery; lienalis; splenic artery; spleen; pancreas; atardamar</t>
-  </si>
-  <si>
-    <t>A. lienalis, dalak ve pankreası besleyen arterlerden biridir.</t>
-  </si>
-  <si>
-    <t>["Bu damar truncus coeliacusun dallarından biridir.","Dalak dokusuna kan taşır.","Pankreasın bir bölümünün beslenmesine katkı sağlar."]</t>
-  </si>
-  <si>
-    <t>mesenterica_superior</t>
-  </si>
-  <si>
-    <t>A. mesenterica superior</t>
-  </si>
-  <si>
-    <t>artery; mesenterica superior; superior mesenteric artery; intestine; atardamar</t>
-  </si>
-  <si>
-    <t>A. mesenterica superior, ince bağırsak ve kalın bağırsağın bir bölümünü besleyen arterdir.</t>
-  </si>
-  <si>
-    <t>["Bu damar karın aortundan ayrılır.","İnce bağırsağa kan taşır.","Kalın bağırsağın ilk yarısının beslenmesine katkı sağlar."]</t>
-  </si>
-  <si>
-    <t>mesenterica_inferior</t>
-  </si>
-  <si>
-    <t>A. mesenterica inferior</t>
-  </si>
-  <si>
-    <t>artery; mesenterica inferior; inferior mesenteric artery; intestine; atardamar</t>
-  </si>
-  <si>
-    <t>A. mesenterica inferior, kalın bağırsağın ikinci yarısını besleyen arterdir.</t>
-  </si>
-  <si>
-    <t>["Bu damar karın aortundan ayrılır.","Kalın bağırsağın alt bölümlerine kan taşır.","Sindirim sisteminin alt kısmının beslenmesinde görev alır."]</t>
-  </si>
-  <si>
-    <t>renalis</t>
-  </si>
-  <si>
-    <t>A. renalis</t>
-  </si>
-  <si>
-    <t>artery; renalis; renal artery; kidney; atardamar</t>
-  </si>
-  <si>
-    <t>A. renalis, böbreklere kan taşıyan büyük arterlerden biridir.</t>
-  </si>
-  <si>
-    <t>["Bu damar karın aortundan ayrılır.","Böbreklere oksijen bakımından zengin kan taşır.","Böbrek dokusunun beslenmesinde önemli rol oynar."]</t>
-  </si>
-  <si>
-    <t>gonadal_artery</t>
-  </si>
-  <si>
-    <t>A. testicularis / A. ovarica</t>
-  </si>
-  <si>
-    <t>artery; testicular artery; ovarian artery; gonadal artery; atardamar</t>
-  </si>
-  <si>
-    <t>A. testicularis ve A. ovarica, üreme organlarını besleyen arterlerdir.</t>
-  </si>
-  <si>
-    <t>["Bu damarlar karın aortundan ayrılır.","Erkeklerde testislerin kanlanmasını sağlar.","Kadınlarda yumurtalıkların beslenmesinde görev alır."]</t>
-  </si>
-  <si>
-    <t>lumbales</t>
-  </si>
-  <si>
-    <t>A. lumbales</t>
-  </si>
-  <si>
-    <t>artery; lumbales; lumbar artery; spine; atardamar</t>
-  </si>
-  <si>
-    <t>A. lumbales, bel bölgesindeki yapıları besleyen arterlerdir.</t>
-  </si>
-  <si>
-    <t>["Bu damarlar karın aortundan ayrılır.","Omurilik çevresindeki kas ve dokulara kan taşırlar.","Bel bölgesinin kanlanmasına katkı sağlarlar."]</t>
-  </si>
-  <si>
-    <t>sacralis_media</t>
-  </si>
-  <si>
-    <t>A. sacralis media</t>
-  </si>
-  <si>
-    <t>artery; sacralis media; sacral artery; sacrum; atardamar</t>
-  </si>
-  <si>
-    <t>A. sacralis media, sakrum bölgesini besleyen arterdir.</t>
-  </si>
-  <si>
-    <t>["Bu damar karın aortunun alt kısmından ayrılır.","Sakrum bölgesine kan taşır.","Pelvis bölgesindeki bazı yapıların beslenmesine katkı sağlar."]</t>
-  </si>
-  <si>
-    <t>phrenica_inferior</t>
-  </si>
-  <si>
-    <t>A. phrenica inferior</t>
-  </si>
-  <si>
-    <t>artery; phrenica inferior; inferior phrenic artery; diaphragm; atardamar</t>
-  </si>
-  <si>
-    <t>A. phrenica inferior, diyaframın alt kısmını besleyen arterlerden biridir.</t>
-  </si>
-  <si>
-    <t>["Bu damar karın aortundan ayrılır.","Diyaframın alt yüzüne kan taşır.","Diyafram kasının beslenmesinde görev alır."]</t>
-  </si>
-  <si>
-    <t>iliaca_communis</t>
-  </si>
-  <si>
-    <t>A. iliaca communis</t>
-  </si>
-  <si>
-    <t>Lower_Extremity</t>
-  </si>
-  <si>
-    <t>artery; iliaca communis; common iliac artery; pelvis; atardamar</t>
-  </si>
-  <si>
-    <t>A. iliaca communis, karın aortunun ikiye ayrılmasıyla oluşan büyük arterlerden biridir.</t>
-  </si>
-  <si>
-    <t>["Karın aortu yaklaşık dördüncü bel omuru hizasında ikiye ayrılarak sağ ve sol a. iliaca communis arterlerini oluşturur.","Bu arter pelvis bölgesine doğru ilerler.","Pelvis içinde a. iliaca interna ve a. iliaca externa olmak üzere iki ana dala ayrılır."]</t>
-  </si>
-  <si>
-    <t>Ders kitabı s.139</t>
-  </si>
-  <si>
-    <t>iliaca_interna</t>
-  </si>
-  <si>
-    <t>A. iliaca interna</t>
-  </si>
-  <si>
-    <t>artery; iliaca interna; internal iliac artery; pelvis; atardamar</t>
-  </si>
-  <si>
-    <t>A. iliaca interna, pelvis boşluğundaki organları besleyen arterdir.</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> ["Bu damar a. iliaca communis'in dallarından biridir.","Pelvis boşluğu içinde ilerler.","Mesane, rektum ve pelvis kasları gibi yapılara dallar vererek bu bölgelerin beslenmesini sağlar."]</t>
-  </si>
-  <si>
-    <t>iliaca_externa</t>
-  </si>
-  <si>
-    <t>A. iliaca externa</t>
-  </si>
-  <si>
-    <t>artery; iliaca externa; external iliac artery; leg; atardamar</t>
-  </si>
-  <si>
-    <t>A. iliaca externa, alt ekstremiteye kan taşıyan önemli arterlerden biridir.</t>
-  </si>
-  <si>
-    <t>["Bu damar a. iliaca communis'in iki ana dalından biridir.","Pelvis bölgesinden çıkarak bacaklara doğru ilerler.","Alt ekstremitenin kanlanmasını sağlayan arteriyel dolaşımın devamını oluşturur."]</t>
-  </si>
-  <si>
-    <t>femoralis</t>
-  </si>
-  <si>
-    <t>A. femoralis</t>
-  </si>
-  <si>
-    <t>artery; femoralis; femoral artery; thigh; atardamar</t>
-  </si>
-  <si>
-    <t>A. femoralis, uyluk bölgesini besleyen büyük bir arterdir.</t>
-  </si>
-  <si>
-    <t>["A. iliaca externa uyluk bölgesine ulaştığında a. femoralis adını alır.","Bu arter uyluk kaslarına dallar vererek bölgenin kanlanmasını sağlar.","Uyluk boyunca aşağı doğru ilerleyerek diz bölgesine ulaşır."]</t>
-  </si>
-  <si>
-    <t>poplitea</t>
-  </si>
-  <si>
-    <t>A. poplitea</t>
-  </si>
-  <si>
-    <t>artery; poplitea; popliteal artery; knee; atardamar</t>
-  </si>
-  <si>
-    <t>A. poplitea, diz arkasında bulunan ve diz bölgesini besleyen arterdir.</t>
-  </si>
-  <si>
-    <t>["A. femoralis diz bölgesine ulaştığında a. poplitea adını alır.","Bu arter dizin arka kısmında yer alır.","Diz çevresindeki yapıların beslenmesini sağlar."]</t>
-  </si>
-  <si>
-    <t>tibialis_anterior</t>
-  </si>
-  <si>
-    <t>A. tibialis anterior</t>
-  </si>
-  <si>
-    <t>artery; tibialis anterior; anterior tibial artery; leg; atardamar</t>
-  </si>
-  <si>
-    <t>A. tibialis anterior, bacağın ön kısmını besleyen arterdir.</t>
-  </si>
-  <si>
-    <t>["A. poplitea baldır bölgesinde iki ana dala ayrılır.","Bu dallardan biri a. tibialis anteriordur.","Bacağın ön kısmındaki kasların ve dokuların beslenmesini sağlar.","Ayak sırtında a. dorsalis pedis olarak devam eder."]</t>
-  </si>
-  <si>
-    <t>tibialis_posterior</t>
-  </si>
-  <si>
-    <t>A. tibialis posterior</t>
-  </si>
-  <si>
-    <t>artery; tibialis posterior; posterior tibial artery; leg; atardamar</t>
-  </si>
-  <si>
-    <t>A. tibialis posterior, bacağın arka bölümünü besleyen arterdir.</t>
-  </si>
-  <si>
-    <t>["A. poplitea baldır bölgesinde a. tibialis anterior ve a. tibialis posterior olarak ikiye ayrılır.","A. tibialis posterior bacağın arka bölümündeki kasları besler.","Alt bacak ve ayak bölgesinin kanlanmasına katkı sağlar."]</t>
-  </si>
-  <si>
-    <t>dorsalis_pedis</t>
-  </si>
-  <si>
-    <t>A. dorsalis pedis</t>
-  </si>
-  <si>
-    <t>artery; dorsalis pedis; foot artery; pulse; atardamar</t>
-  </si>
-  <si>
-    <t>A. dorsalis pedis, ayağın üst kısmında bulunan arterdir.</t>
-  </si>
-  <si>
-    <t>["A. tibialis anterior ayak sırtına ulaştığında a. dorsalis pedis adını alır.","Ayağın üst kısmındaki dokuların beslenmesini sağlar.","Birinci metatarsal aralıkta bu arter üzerinden nabız alınabilir."]</t>
-  </si>
-  <si>
-    <t>temporalis</t>
-  </si>
-  <si>
-    <t>A. temporalis</t>
-  </si>
-  <si>
-    <t>Head_Face</t>
-  </si>
-  <si>
-    <t>artery; temporalis; temporal artery; nabız; atardamar</t>
-  </si>
-  <si>
-    <t>A. temporalis, baş bölgesinde nabız alınabilen arterlerden biridir.</t>
-  </si>
-  <si>
-    <t>["Bu arter şakak bölgesinde bulunur.","Baş bölgesinde nabız değerlendirilirken bu damardan yararlanılabilir."]</t>
-  </si>
-  <si>
-    <t>Ders kitabı s.143</t>
-  </si>
-  <si>
-    <t>carotis_communis</t>
-  </si>
-  <si>
-    <t>A. carotis communis</t>
-  </si>
-  <si>
-    <t>Neck</t>
-  </si>
-  <si>
-    <t>artery; carotis communis; carotid artery; nabız; atardamar</t>
-  </si>
-  <si>
-    <t>A. carotis communis, boyun bölgesinde nabız alınabilen önemli arterlerden biridir.</t>
-  </si>
-  <si>
-    <t>["Bu arter boyunda yer alır.","Fiziksel muayenede karotis arterden nabız alınabilir.","Karotis arterden nabız alınırken dikkat edilmelidir."]</t>
-  </si>
-  <si>
-    <t>axillaris_pulse</t>
-  </si>
-  <si>
-    <t>artery; axillaris; axillary artery; nabız; atardamar</t>
-  </si>
-  <si>
-    <t>A. axillaris, üst ekstremitede nabız alınabilen arterlerden biridir.</t>
-  </si>
-  <si>
-    <t>["Bu arter koltuk altı bölgesinde bulunur.","Üst ekstremite arterlerinden biri olarak nabız değerlendirmesinde kullanılabilir."]</t>
-  </si>
-  <si>
-    <t>brachialis_pulse</t>
-  </si>
-  <si>
-    <t>artery; brachialis; brachial artery; nabız; atardamar</t>
-  </si>
-  <si>
-    <t>A. brachialis, üst ekstremitede nabız alınabilen arterlerden biridir.</t>
-  </si>
-  <si>
-    <t>["Bu arter kol bölgesinde bulunur.","Fiziksel muayenede üst ekstremite arterlerinden biri olarak nabız değerlendirilmesinde kullanılabilir."]</t>
-  </si>
-  <si>
-    <t>ulnaris_pulse</t>
-  </si>
-  <si>
-    <t>artery; ulnaris; ulnar artery; nabız; atardamar</t>
-  </si>
-  <si>
-    <t>A. ulnaris, ön kol bölgesinde bulunan arterlerden biridir.</t>
-  </si>
-  <si>
-    <t>["Bu arter ön kol bölgesinde yer alır.","Üst ekstremitede nabız alınabilen arterlerden biridir."]</t>
-  </si>
-  <si>
-    <t>radialis_pulse</t>
-  </si>
-  <si>
-    <t>artery; radialis; radial artery; nabız; atardamar</t>
-  </si>
-  <si>
-    <t>A. radialis, el bileğinde nabız alınmasında yaygın olarak kullanılan arterdir.</t>
-  </si>
-  <si>
-    <t>["Bu arter el bileği bölgesinde bulunur.","Rutin muayenelerde nabız genellikle radial arter üzerinden değerlendirilir."]</t>
-  </si>
-  <si>
-    <t>femoralis_pulse</t>
-  </si>
-  <si>
-    <t>artery; femoralis; femoral artery; nabız; atardamar</t>
-  </si>
-  <si>
-    <t>A. femoralis, alt ekstremitede nabız alınabilen arterlerden biridir.</t>
-  </si>
-  <si>
-    <t>["Bu arter uyluk bölgesinde bulunur.","Alt ekstremite arterlerinden biri olarak nabız değerlendirilmesinde kullanılabilir."]</t>
-  </si>
-  <si>
-    <t>poplitea_pulse</t>
-  </si>
-  <si>
-    <t>artery; poplitea; popliteal artery; nabız; atardamar</t>
-  </si>
-  <si>
-    <t>A. poplitea, diz arkasında bulunan arterdir.</t>
-  </si>
-  <si>
-    <t>["Bu arter dizin arka kısmında yer alır.","Alt ekstremitede nabız değerlendirilirken bu damardan yararlanılabilir."]</t>
-  </si>
-  <si>
-    <t>tibialis_posterior_pulse</t>
-  </si>
-  <si>
-    <t>artery; tibialis posterior; posterior tibial artery; nabız; atardamar</t>
-  </si>
-  <si>
-    <t>A. tibialis posterior, alt bacak bölgesinde nabız alınabilen arterlerden biridir.</t>
-  </si>
-  <si>
-    <t>["Bu arter baldır bölgesinde yer alır.","Alt ekstremitede nabız değerlendirilmesinde kullanılan arterlerden biridir."]</t>
-  </si>
-  <si>
-    <t>dorsalis_pedis_pulse</t>
-  </si>
-  <si>
-    <t>Foot</t>
-  </si>
-  <si>
-    <t>artery; dorsalis pedis; foot artery; nabız; atardamar</t>
-  </si>
-  <si>
-    <t>["Bu arter ayak sırtında bulunur.","Alt ekstremitede nabız değerlendirilirken bu damardan yararlanılabilir."]</t>
-  </si>
-  <si>
-    <t>veins</t>
-  </si>
-  <si>
-    <t>Toplardamarlar</t>
-  </si>
-  <si>
-    <t>vein; vena; ven; circulation; toplardamar</t>
-  </si>
-  <si>
-    <t>Toplardamarlar, kanı dokular ve akciğerlerden kalbe taşıyan damar grubudur.</t>
-  </si>
-  <si>
-    <t>["Temiz kanı akciğerlerden kalbe taşıyan akciğer toplardamarları dışında venler kirli kan taşır.","Venlerde kan basıncı arterlere göre daha düşüktür.","Ven duvarları arterlere göre daha incedir.","Normal istirahat halinde dolaşımdaki kanın büyük bir bölümü venlerde bulunur."]</t>
-  </si>
-  <si>
-    <t>Ders kitabı s.140</t>
-  </si>
-  <si>
-    <t>upper_extremity_veins</t>
-  </si>
-  <si>
-    <t>Üst ekstremite venleri</t>
-  </si>
-  <si>
-    <t>vein; upper extremity veins; arm veins; vena; toplardamar</t>
-  </si>
-  <si>
-    <t>Üst ekstremite venleri, kol bölgesindeki kirli kanı kalbe doğru taşıyan toplardamarlardır.</t>
-  </si>
-  <si>
-    <t>["Üst ekstremite venleri yüzeysel ve derin venler olmak üzere iki grupta incelenir.","Yüzeysel venler deri altında seyreder ve görülebilir.","Önemli yüzeysel venler arasında v. cephalica, v. basilica, v. mediana antebrachii ve v. mediana cubiti bulunur.","Derin venler arterlerle birlikte seyreder.","Önemli derin venler arasında v. radialis, v. ulnaris, v. brachialis ve v. axillaris yer alır.","Üst ekstremiteden gelen venöz kan v. subclavia üzerinden daha büyük venlere taşınır."]</t>
-  </si>
-  <si>
-    <t>brachiocephalica_vein</t>
-  </si>
-  <si>
-    <t>V. brachiocephalica</t>
-  </si>
-  <si>
-    <t>vein; brachiocephalica; brachiocephalic vein; toplardamar</t>
-  </si>
-  <si>
-    <t>V. brachiocephalica, kol ve baş bölgesinden gelen venlerin birleşmesi ile oluşur.</t>
-  </si>
-  <si>
-    <t>["Baş bölgesinden gelen v. jugularis interna ile boynun dış venlerinden v. jugularis externa birleşir.","Koldan gelen v. subclavia ile birleşerek v. brachiocephalica oluşur."]</t>
-  </si>
-  <si>
-    <t>jugularis_interna</t>
-  </si>
-  <si>
-    <t>V. jugularis interna</t>
-  </si>
-  <si>
-    <t>vein; jugularis interna; internal jugular vein; toplardamar</t>
-  </si>
-  <si>
-    <t>V. jugularis interna boyundaki en büyük vendir.</t>
-  </si>
-  <si>
-    <t>["El sırtının ulnar tarafından başlar.","Ön kolun iç yüzünden yukarı doğru ilerler.","Dirsek bölgesini geçerek kol bölgesine ulaşır.","Kol bölgesinde derine ilerler ve derin venöz sistemle birleşerek v. axillaris'in oluşumuna katılır."]</t>
-  </si>
-  <si>
-    <t>jugularis_externa</t>
-  </si>
-  <si>
-    <t>V. jugularis externa</t>
-  </si>
-  <si>
-    <t>vein; jugularis externa; external jugular vein; toplardamar</t>
-  </si>
-  <si>
-    <t>V. jugularis externa başın dış venlerini ve yüzün yüzeysel venlerini toplar.</t>
-  </si>
-  <si>
-    <t>["Baş ve yüzün yüzeysel venleri ile birleşir.","Boyundan aşağı doğru ilerler.","V. subclavia ile birleşerek sonlanır."]</t>
-  </si>
-  <si>
-    <t>subclavia_vein</t>
-  </si>
-  <si>
-    <t>V. subclavia</t>
-  </si>
-  <si>
-    <t>vein; subclavia; subclavian vein; toplardamar</t>
-  </si>
-  <si>
-    <t>V. subclavia, v. axillaris'in köprücük kemiği altındaki devamı olan vendir.</t>
-  </si>
-  <si>
-    <t>["Kol venleri birleşerek v. axillaris'i oluşturur.","V. axillaris köprücük kemiğinin altında v. subclavia adını alır.","Buradan jugular venlerle birleşerek v. brachiocephalica'yı oluşturur."]</t>
-  </si>
-  <si>
-    <t>axillaris_vein</t>
-  </si>
-  <si>
-    <t>V. axillaris</t>
-  </si>
-  <si>
-    <t>vein; axillaris; axillary vein; toplardamar</t>
-  </si>
-  <si>
-    <t>V. axillaris, üst ekstremitenin derin venöz dönüşünde yer alan ve koltuk altı bölgesinde bulunan büyük bir vendir.</t>
-  </si>
-  <si>
-    <t>["Kol bölgesindeki venlerin birleşmesi ile oluşur.","Koltuk altı bölgesinde bulunur.","Yukarı doğru ilerleyerek v. subclavia olarak devam eder."]</t>
-  </si>
-  <si>
-    <t>cephalica_vein</t>
-  </si>
-  <si>
-    <t>V. cephalica</t>
-  </si>
-  <si>
-    <t>vein; cephalica; cephalic vein; toplardamar</t>
-  </si>
-  <si>
-    <t>V. cephalica üst ekstremitenin önemli yüzeysel venlerinden biridir.</t>
-  </si>
-  <si>
-    <t>["El sırtının radyal tarafından başlar.","Ön kolun ön tarafına doğru ilerler.","Kolun dış yanından yukarı çıkar.","Proksimalde v. axillaris'e katılır."]</t>
-  </si>
-  <si>
-    <t>brachialis_vein</t>
-  </si>
-  <si>
-    <t>V. brachialis</t>
-  </si>
-  <si>
-    <t>vein; brachialis; brachial vein; toplardamar</t>
-  </si>
-  <si>
-    <t>V. brachialis kol bölgesinin derin venlerinden biridir.</t>
-  </si>
-  <si>
-    <t>["V. radialis ve v. ulnaris'in dirsek önünde birleşmesi ile oluşur.","Yukarı doğru ilerleyerek v. axillaris'e katılır."]</t>
-  </si>
-  <si>
-    <t>basilica_vein</t>
-  </si>
-  <si>
-    <t>V. basilica</t>
-  </si>
-  <si>
-    <t>vein; basilica; basilic vein; toplardamar</t>
-  </si>
-  <si>
-    <t>V. basilica üst ekstremitenin önemli yüzeysel venlerinden biridir.</t>
-  </si>
-  <si>
-    <t>mediana_cubiti</t>
-  </si>
-  <si>
-    <t>V. mediana cubiti</t>
-  </si>
-  <si>
-    <t>vein; mediana cubiti; median cubital vein; toplardamar</t>
-  </si>
-  <si>
-    <t>V. mediana cubiti dirsek bölgesinde bulunan yüzeysel vendir.</t>
-  </si>
-  <si>
-    <t>["Dirsek ekleminin iç yüzünde bulunur.","V. basilica ile v. cephalica'yı birbirine bağlar."]</t>
-  </si>
-  <si>
-    <t>antebrachii_mediana</t>
-  </si>
-  <si>
-    <t>V. antebrachii mediana</t>
-  </si>
-  <si>
-    <t>vein; antebrachii mediana; median antebrachial vein; toplardamar</t>
-  </si>
-  <si>
-    <t>V. antebrachii mediana ön kolun yüzeysel venlerinden biridir.</t>
-  </si>
-  <si>
-    <t>["Elin palmar yüzünden başlayarak yukarı doğru uzanır.","V. mediana cubiti veya v. basilica ile birleşir."]</t>
-  </si>
-  <si>
-    <t>radialis_vein</t>
-  </si>
-  <si>
-    <t>V. radialis</t>
-  </si>
-  <si>
-    <t>vein; radialis; radial vein; toplardamar</t>
-  </si>
-  <si>
-    <t>V. radialis el ve ön kolun radyal bölgesinin venöz kanını toplar.</t>
-  </si>
-  <si>
-    <t>["El ve ön kolun radyal tarafındaki kirli kanı toplar.","V. ulnaris ile birleşerek v. brachialisi oluşturur."]</t>
-  </si>
-  <si>
-    <t>ulnaris_vein</t>
-  </si>
-  <si>
-    <t>V. ulnaris</t>
-  </si>
-  <si>
-    <t>vein; ulnaris; ulnar vein; toplardamar</t>
-  </si>
-  <si>
-    <t>V. ulnaris el ve ön kolun ulnar bölgesinin venöz kanını toplar.</t>
-  </si>
-  <si>
-    <t>["El ve ön kolun ulnar tarafındaki kirli kanı toplar.","V. radialis ile birleşerek v. brachialisi oluşturur."]</t>
-  </si>
-  <si>
-    <t>cava_superior</t>
-  </si>
-  <si>
-    <t>V. cava superior</t>
-  </si>
-  <si>
-    <t>Thorax</t>
-  </si>
-  <si>
-    <t>vein; cava superior; superior vena cava; toplardamar</t>
-  </si>
-  <si>
-    <t>V. cava superior, baş, boyun, göğüs ve üst ekstremite bölgelerinden gelen venöz kanı kalbe taşıyan büyük bir toplardamardır.</t>
-  </si>
-  <si>
-    <t>["V. cava superior iki adet v. brachiocephalicanın birleşmesi ile oluşur.","Baş, boyun, göğüs ve üst ekstremite bölgelerinden gelen kirli kanı toplar.","Topladığı kanı kalbin sağ atriumuna taşır."]</t>
-  </si>
-  <si>
-    <t>lower_extremity_veins</t>
-  </si>
-  <si>
-    <t>Alt ekstremite venleri</t>
-  </si>
-  <si>
-    <t>vein; lower extremity veins; leg veins; vena; toplardamar</t>
-  </si>
-  <si>
-    <t>Alt ekstremite venleri bacak ve ayak bölgesindeki venöz kanı kalbe doğru taşıyan toplardamarlardır.</t>
-  </si>
-  <si>
-    <t>["Alt ekstremite venleri yüzeysel ve derin venler olmak üzere iki grupta incelenir.","Yüzeysel venlerin yapısında kapakçıklar bulunur.","Derin venler genellikle aynı isimdeki arterlerle birlikte seyreder.","Alt ekstremiteden gelen venöz kan daha büyük venler aracılığıyla v. cava inferiora taşınır."]</t>
-  </si>
-  <si>
-    <t>Ders kitabı s.141</t>
-  </si>
-  <si>
-    <t>cava_inferior</t>
-  </si>
-  <si>
-    <t>V. cava inferior</t>
-  </si>
-  <si>
-    <t>vein; cava inferior; inferior vena cava; toplardamar</t>
-  </si>
-  <si>
-    <t>V. cava inferior gövdenin alt bölümünden gelen venöz kanı kalbe taşıyan büyük bir vendir.</t>
-  </si>
-  <si>
-    <t>["Gövdede diyaframın altında kalan bölüm ile alt ekstremite bölgelerinin kanını toplar.","Sağ ve sol v. iliaca communis'in birleşmesi ile oluşur.","Topladığı kanı kalbin sağ atriumuna taşır."]</t>
-  </si>
-  <si>
-    <t>iliaca_communis_vein</t>
-  </si>
-  <si>
-    <t>V. iliaca communis</t>
-  </si>
-  <si>
-    <t>Pelvis</t>
-  </si>
-  <si>
-    <t>vein; iliaca communis; common iliac vein; toplardamar</t>
-  </si>
-  <si>
-    <t>V. iliaca communis pelvis ve alt ekstremitenin venöz kanını taşıyan vendir.</t>
-  </si>
-  <si>
-    <t>["V. iliaca interna ve v. iliaca externa venlerinin birleşmesi ile oluşur.","Sağ ve sol v. iliaca communis venleri birleşerek v. cava inferioru oluşturur."]</t>
-  </si>
-  <si>
-    <t>iliaca_externa_vein</t>
-  </si>
-  <si>
-    <t>V. iliaca externa</t>
-  </si>
-  <si>
-    <t>vein; iliaca externa; external iliac vein; toplardamar</t>
-  </si>
-  <si>
-    <t>V. iliaca externa alt ekstremitenin venöz kanını taşıyan önemli venlerden biridir.</t>
-  </si>
-  <si>
-    <t>["Alt ekstremiteden gelen venöz kanı taşır.","Kasık bölgesinden aşağıda v. femoralis adını alır."]</t>
-  </si>
-  <si>
-    <t>femoralis_vein</t>
-  </si>
-  <si>
-    <t>V. femoralis</t>
-  </si>
-  <si>
-    <t>vein; femoralis; femoral vein; toplardamar</t>
-  </si>
-  <si>
-    <t>V. femoralis bacak bölgesinin venöz kanını taşıyan önemli derin vendir.</t>
-  </si>
-  <si>
-    <t>["Bacak bölgesinin kirli kanını taşır.","V. popliteanın devamıdır.","Yukarı doğru ilerleyerek kasık bölgesinde v. iliaca externa adını alır."]</t>
-  </si>
-  <si>
-    <t>poplitea_vein</t>
-  </si>
-  <si>
-    <t>V. poplitea</t>
-  </si>
-  <si>
-    <t>vein; poplitea; popliteal vein; toplardamar</t>
-  </si>
-  <si>
-    <t>V. poplitea diz arkasında bulunan derin vendir.</t>
-  </si>
-  <si>
-    <t>["V. tibialis anterior ve v. tibialis posteriorun birleşmesi ile oluşur.","Diz arkasından yukarı doğru ilerler.","Yukarıda v. femoralis adını alır."]</t>
-  </si>
-  <si>
-    <t>tibialis_anterior_vein</t>
-  </si>
-  <si>
-    <t>V. tibialis anterior</t>
-  </si>
-  <si>
-    <t>vein; tibialis anterior; anterior tibial vein; toplardamar</t>
-  </si>
-  <si>
-    <t>V. tibialis anterior ayak ve bacağın ön bölümünden gelen venöz kanı taşır.</t>
-  </si>
-  <si>
-    <t>["Ayak sırtından başlayarak baldırın önünden yukarı doğru ilerler.","V. tibialis posterior ile birleşerek v. popliteayı oluşturur."]</t>
-  </si>
-  <si>
-    <t>tibialis_posterior_vein</t>
-  </si>
-  <si>
-    <t>V. tibialis posterior</t>
-  </si>
-  <si>
-    <t>vein; tibialis posterior; posterior tibial vein; toplardamar</t>
-  </si>
-  <si>
-    <t>V. tibialis posterior ayak tabanı ve baldır bölgesinin venöz kanını taşır.</t>
-  </si>
-  <si>
-    <t>["Ayak tabanından başlayarak baldırın arka kısmından yukarı doğru ilerler.","V. tibialis anterior ile birleşerek v. popliteayı oluşturur."]</t>
-  </si>
-  <si>
-    <t>saphena_magna</t>
-  </si>
-  <si>
-    <t>V. saphena magna</t>
-  </si>
-  <si>
-    <t>vein; saphena magna; great saphenous vein; toplardamar</t>
-  </si>
-  <si>
-    <t>V. saphena magna vücudun en uzun venidir.</t>
-  </si>
-  <si>
-    <t>["Ayak sırtından başlar.","Bacağın iç yüzünden yukarı doğru ilerler.","Kasık bölgesinde v. femoralis ile birleşir.","Koroner arter bypass ameliyatlarında greft olarak kullanılabilir."]</t>
-  </si>
-  <si>
-    <t>saphena_parva</t>
-  </si>
-  <si>
-    <t>V. saphena parva</t>
-  </si>
-  <si>
-    <t>vein; saphena parva; small saphenous vein; toplardamar</t>
-  </si>
-  <si>
-    <t>V. saphena parva alt ekstremitenin yüzeysel venlerinden biridir.</t>
-  </si>
-  <si>
-    <t>["Ayak sırtının dış tarafından başlar.","Baldırın arka kısmından yukarı doğru ilerler.","Diz arkasında derine ilerleyerek v. popliteaya bağlanır."]</t>
-  </si>
-  <si>
-    <t>systemic_circulation</t>
-  </si>
-  <si>
-    <t>Büyük kan dolaşımı</t>
-  </si>
-  <si>
-    <t>Circulation</t>
-  </si>
-  <si>
-    <t>circulation; systemic; large_circulation; heart; body</t>
-  </si>
-  <si>
-    <t>Büyük kan dolaşımı, oksijen bakımından zengin kanın kalpten çıkarak tüm vücut dokularına gönderilmesini ve dokularda oluşan karbondioksit ile atık maddelerin toplanarak tekrar kalbe getirilmesini sağlayan dolaşımdır.</t>
-  </si>
-  <si>
-    <t>["Oksijenlenmiş kan pulmoner venler ile sol atriyuma gelir", "Kan mitral kapaktan geçerek sol ventriküle ulaşır", "Sol ventrikül kasılarak kanı aort aracılığıyla tüm vücuda pompalar", "Dokularda gaz değişimi gerçekleşir ve kan kirlenir", "Kirli kan vena cava damarları ile sağ atriyuma geri döner"]</t>
-  </si>
-  <si>
-    <t>Ders kitabı s.145</t>
-  </si>
-  <si>
-    <t>pulmonary_circulation</t>
-  </si>
-  <si>
-    <t>Küçük kan dolaşımı</t>
-  </si>
-  <si>
-    <t>circulation; pulmonary; small_circulation; heart; lung</t>
-  </si>
-  <si>
-    <t>Küçük kan dolaşımı, kalpten akciğerlere gönderilen kirli kanın akciğerlerde oksijenlenerek temizlenmesi ve tekrar kalbe dönmesini sağlayan dolaşımdır.</t>
-  </si>
-  <si>
-    <t>["Kirli kan sağ atriyuma gelir", "Kan triküspit kapaktan geçerek sağ ventriküle ulaşır", "Sağ ventrikül kasılarak kanı pulmoner arter aracılığıyla akciğerlere pompalar", "Akciğerlerde gaz değişimi gerçekleşir ve kan oksijenlenir", "Oksijenlenmiş kan pulmoner venler ile sol atriyuma geri döner"]</t>
-  </si>
-  <si>
-    <t>systemic_left_ventricle_01</t>
-  </si>
-  <si>
-    <t>Sol ventrikül</t>
-  </si>
-  <si>
-    <t>circulation; systemic; large_circulation; heart; ventricle</t>
-  </si>
-  <si>
-    <t>Sol ventrikül, oksijen bakımından zengin kanı aort aracılığıyla tüm vücuda pompalayan ve büyük kan dolaşımının başladığı kalp odacığıdır.</t>
-  </si>
-  <si>
-    <t>["Sol atriyumdan gelen oksijenli kan sol ventrikülde toplanır", "Ventrikül kasılarak kanı kalpten dışarı pompalar", "Kan aort damarına gönderilir"]</t>
-  </si>
-  <si>
-    <t>systemic_aorta_02</t>
-  </si>
-  <si>
     <t>circulation; systemic; large_circulation; vessel; artery; aorta</t>
   </si>
   <si>
@@ -1426,7 +1429,7 @@
     <t>systemic_body_arteries_03</t>
   </si>
   <si>
-    <t>Vücut atardamarları</t>
+    <t>Arteriae corporis</t>
   </si>
   <si>
     <t>circulation; systemic; large_circulation; vessel; artery; systemic_artery</t>
@@ -1441,13 +1444,13 @@
     <t>systemic_capillaries_04</t>
   </si>
   <si>
-    <t>Vücut kılcal damarları</t>
+    <t>Vasa capillaria corporis</t>
   </si>
   <si>
     <t>circulation; systemic; large_circulation; capillary; body</t>
   </si>
   <si>
-    <t>Kılcal damarlar, kan ile hücreler arasında gaz ve madde alışverişinin gerçekleştiği en ince damarlardır.</t>
+    <t>Vasa capillaria, kan ile hücreler arasında gaz ve madde alışverişinin gerçekleştiği en ince damarlardır.</t>
   </si>
   <si>
     <t>["Oksijenli kan kılcal damarlara ulaşır", "Hücreler oksijeni ve besin maddelerini alır", "Karbondioksit ve atık maddeler kana geçer" , "Kan kirli hale gelir"]</t>
@@ -1456,13 +1459,13 @@
     <t>systemic_body_veins_05</t>
   </si>
   <si>
-    <t>Vücut toplardamarları</t>
+    <t>Venae corporis</t>
   </si>
   <si>
     <t>circulation; systemic; large_circulation; vein; body</t>
   </si>
   <si>
-    <t>Toplardamarlar, dokularda gaz değişimi sonucu kirlenen kanı kılcal damarlardan alarak kalbe doğru taşıyan damarlardır.</t>
+    <t>Venler, dokularda gaz değişimi sonucu kirlenen kanı kılcal damarlardan alarak kalbe doğru taşıyan damarlardır.</t>
   </si>
   <si>
     <t>["Kılcal damarlardan çıkan kirli kan küçük toplardamarlara geçer", "Toplardamarlar birleşerek daha büyük damarları oluşturur", "Kan kalbe doğru taşınır"]</t>
@@ -1480,7 +1483,7 @@
     <t>Vena cava superior ve vena cava inferior, vücuttan gelen kirli kanı kalbin sağ atriyumuna taşıyan büyük toplardamarlardır.</t>
   </si>
   <si>
-    <t>["Vücuttan gelen kirli kan büyük toplardamarlarda toplanır", "Kan vena cava damarlarına ulaşır", "Vena cava kanı kalbin sağ atriyumuna taşır"]</t>
+    <t>["Vücuttan gelen kirli kan büyük toplardamarlarda toplanır", "Kan vena cava'ya ulaşır", "V. cava superior ve V. cava inferior kanı sağ atriyuma taşır."]</t>
   </si>
   <si>
     <t>systemic_right_atrium_07</t>
@@ -1492,10 +1495,10 @@
     <t>circulation; systemic; large_circulation; heart; atrium</t>
   </si>
   <si>
-    <t>Sağ atriyum, vena cava damarları aracılığıyla vücuttan gelen kirli kanın toplandığı kalp odacığıdır.</t>
-  </si>
-  <si>
-    <t>["Vena cava damarlarından gelen kan sağ atriyuma ulaşır", "Sağ atriyum kanı sağ ventriküle iletmeye hazır hale getirir"]</t>
+    <t>Sağ atriyum, vena cava aracılığıyla vücuttan gelen kirli kanın toplandığı kalp odacığıdır.</t>
+  </si>
+  <si>
+    <t>["Vena cava'dan gelen kan sağ atriyuma ulaşır", "Sağ atriyum kanı sağ ventriküle iletmeye hazır hale getirir"]</t>
   </si>
   <si>
     <t>pulmonary_right_ventricle_01</t>
@@ -1516,43 +1519,40 @@
     <t>pulmonary_artery_02</t>
   </si>
   <si>
-    <t>Pulmoner arter (A. pulmonalis)</t>
+    <t>A. pulmonalis</t>
   </si>
   <si>
     <t>circulation; pulmonary; small_circulation; vessel; artery; pulmonary_artery</t>
   </si>
   <si>
-    <t>Pulmoner arter, kirli kanı kalpten akciğerlere taşıyan atardamardır.</t>
-  </si>
-  <si>
-    <t>["Sağ ventrikülden çıkan kirli kan pulmoner artere ulaşır", "Pulmoner arter kanı akciğerlere taşır", "Kan akciğer kılcal damarlarına doğru ilerler"]</t>
+    <t>A. pulmonalis, kirli kanı kalpten akciğerlere taşıyan atardamardır.</t>
+  </si>
+  <si>
+    <t>["Sağ ventrikülden çıkan kirli kan pulmoner artere ulaşır", "Pulmoner arter kanı akciğerlere taşır", "Kan Vasa capillaria pulmonum'a doğru ilerler"]</t>
   </si>
   <si>
     <t>pulmonary_capillaries_03</t>
   </si>
   <si>
-    <t>Akciğer kılcal damarları</t>
+    <t>Vasa capillaria pulmonum</t>
   </si>
   <si>
     <t>circulation; pulmonary; small_circulation; vessel; capillary; lung_capillary</t>
   </si>
   <si>
-    <t>Akciğer kılcal damarları, kan ile alveoller arasında gaz değişiminin gerçekleştiği damarlardır.</t>
-  </si>
-  <si>
-    <t>["Kirli kan akciğer kılcal damarlarına ulaşır", "Karbondioksit alveollere verilir", "Oksijen kana geçer", "Kan oksijen bakımından zengin hale gelir"]</t>
+    <t>Vasa capillaria pulmonum, kan ile alveoller arasında gaz değişiminin gerçekleştiği damarlardır.</t>
+  </si>
+  <si>
+    <t>["Kirli kan Vasa capillaria pulmonum'a ulaşır", "Karbondioksit alveollere verilir", "Oksijen kana geçer", "Kan oksijen bakımından zengin hale gelir"]</t>
   </si>
   <si>
     <t>pulmonary_vein_04</t>
   </si>
   <si>
-    <t>Pulmoner ven (V. pulmonalis)</t>
-  </si>
-  <si>
     <t>circulation; pulmonary; small_circulation; vessel; vein; pulmonary_vein</t>
   </si>
   <si>
-    <t>Pulmoner ven, akciğerlerde oksijenlenen kanı kalbe taşıyan toplardamardır.</t>
+    <t>V. pulmonales, akciğerlerde oksijenlenen kanı kalbe taşıyan toplardamarlardır.</t>
   </si>
   <si>
     <t>["Akciğerlerde oksijenlenen kan pulmoner venlere geçer", "Pulmoner venler kanı kalbe taşır", "Kan sol atriyuma ulaşır"]</t>
@@ -4985,7 +4985,7 @@
         <v>58</v>
       </c>
       <c r="E91" s="2" t="s">
-        <v>66</v>
+        <v>467</v>
       </c>
       <c r="F91" s="2" t="s">
         <v>16</v>
@@ -4994,13 +4994,13 @@
         <v>451</v>
       </c>
       <c r="H91" s="2" t="s">
-        <v>467</v>
+        <v>468</v>
       </c>
       <c r="I91" s="2" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="J91" s="2" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="K91" s="2" t="s">
         <v>455</v>
@@ -5008,7 +5008,7 @@
     </row>
     <row r="92">
       <c r="A92" s="2" t="s">
-        <v>470</v>
+        <v>471</v>
       </c>
       <c r="B92" s="2" t="s">
         <v>12</v>
@@ -5020,7 +5020,7 @@
         <v>58</v>
       </c>
       <c r="E92" s="2" t="s">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="F92" s="2" t="s">
         <v>16</v>
@@ -5029,13 +5029,13 @@
         <v>451</v>
       </c>
       <c r="H92" s="2" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="I92" s="2" t="s">
-        <v>473</v>
+        <v>474</v>
       </c>
       <c r="J92" s="2" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="K92" s="2" t="s">
         <v>455</v>
@@ -5043,7 +5043,7 @@
     </row>
     <row r="93">
       <c r="A93" s="2" t="s">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="B93" s="2" t="s">
         <v>12</v>
@@ -5055,7 +5055,7 @@
         <v>58</v>
       </c>
       <c r="E93" s="2" t="s">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="F93" s="2" t="s">
         <v>16</v>
@@ -5064,13 +5064,13 @@
         <v>451</v>
       </c>
       <c r="H93" s="2" t="s">
-        <v>477</v>
+        <v>478</v>
       </c>
       <c r="I93" s="2" t="s">
-        <v>478</v>
+        <v>479</v>
       </c>
       <c r="J93" s="2" t="s">
-        <v>479</v>
+        <v>480</v>
       </c>
       <c r="K93" s="2" t="s">
         <v>455</v>
@@ -5078,7 +5078,7 @@
     </row>
     <row r="94">
       <c r="A94" s="2" t="s">
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="B94" s="2" t="s">
         <v>12</v>
@@ -5090,7 +5090,7 @@
         <v>58</v>
       </c>
       <c r="E94" s="2" t="s">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="F94" s="2" t="s">
         <v>16</v>
@@ -5099,13 +5099,13 @@
         <v>451</v>
       </c>
       <c r="H94" s="2" t="s">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="I94" s="2" t="s">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="J94" s="2" t="s">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="K94" s="2" t="s">
         <v>455</v>
@@ -5113,7 +5113,7 @@
     </row>
     <row r="95">
       <c r="A95" s="2" t="s">
-        <v>485</v>
+        <v>486</v>
       </c>
       <c r="B95" s="2" t="s">
         <v>12</v>
@@ -5125,7 +5125,7 @@
         <v>58</v>
       </c>
       <c r="E95" s="2" t="s">
-        <v>486</v>
+        <v>487</v>
       </c>
       <c r="F95" s="2" t="s">
         <v>16</v>
@@ -5134,13 +5134,13 @@
         <v>451</v>
       </c>
       <c r="H95" s="2" t="s">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="I95" s="2" t="s">
-        <v>488</v>
+        <v>489</v>
       </c>
       <c r="J95" s="2" t="s">
-        <v>489</v>
+        <v>490</v>
       </c>
       <c r="K95" s="2" t="s">
         <v>455</v>
@@ -5148,7 +5148,7 @@
     </row>
     <row r="96">
       <c r="A96" s="2" t="s">
-        <v>490</v>
+        <v>491</v>
       </c>
       <c r="B96" s="2" t="s">
         <v>12</v>
@@ -5160,7 +5160,7 @@
         <v>23</v>
       </c>
       <c r="E96" s="2" t="s">
-        <v>491</v>
+        <v>492</v>
       </c>
       <c r="F96" s="2" t="s">
         <v>16</v>
@@ -5169,13 +5169,13 @@
         <v>451</v>
       </c>
       <c r="H96" s="2" t="s">
-        <v>492</v>
+        <v>493</v>
       </c>
       <c r="I96" s="2" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="J96" s="2" t="s">
-        <v>494</v>
+        <v>495</v>
       </c>
       <c r="K96" s="2" t="s">
         <v>455</v>
@@ -5183,7 +5183,7 @@
     </row>
     <row r="97">
       <c r="A97" s="2" t="s">
-        <v>495</v>
+        <v>496</v>
       </c>
       <c r="B97" s="2" t="s">
         <v>12</v>
@@ -5195,7 +5195,7 @@
         <v>23</v>
       </c>
       <c r="E97" s="2" t="s">
-        <v>496</v>
+        <v>497</v>
       </c>
       <c r="F97" s="2" t="s">
         <v>16</v>
@@ -5204,13 +5204,13 @@
         <v>451</v>
       </c>
       <c r="H97" s="2" t="s">
-        <v>497</v>
+        <v>498</v>
       </c>
       <c r="I97" s="2" t="s">
-        <v>498</v>
+        <v>499</v>
       </c>
       <c r="J97" s="2" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="K97" s="2" t="s">
         <v>455</v>
@@ -5218,7 +5218,7 @@
     </row>
     <row r="98">
       <c r="A98" s="2" t="s">
-        <v>500</v>
+        <v>501</v>
       </c>
       <c r="B98" s="2" t="s">
         <v>12</v>
@@ -5230,7 +5230,7 @@
         <v>58</v>
       </c>
       <c r="E98" s="2" t="s">
-        <v>501</v>
+        <v>502</v>
       </c>
       <c r="F98" s="2" t="s">
         <v>16</v>
@@ -5239,13 +5239,13 @@
         <v>451</v>
       </c>
       <c r="H98" s="2" t="s">
-        <v>502</v>
+        <v>503</v>
       </c>
       <c r="I98" s="2" t="s">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="J98" s="2" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="K98" s="2" t="s">
         <v>455</v>
@@ -5253,7 +5253,7 @@
     </row>
     <row r="99">
       <c r="A99" s="2" t="s">
-        <v>505</v>
+        <v>506</v>
       </c>
       <c r="B99" s="2" t="s">
         <v>12</v>
@@ -5265,7 +5265,7 @@
         <v>58</v>
       </c>
       <c r="E99" s="2" t="s">
-        <v>506</v>
+        <v>507</v>
       </c>
       <c r="F99" s="2" t="s">
         <v>16</v>
@@ -5274,13 +5274,13 @@
         <v>451</v>
       </c>
       <c r="H99" s="2" t="s">
-        <v>507</v>
+        <v>508</v>
       </c>
       <c r="I99" s="2" t="s">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="J99" s="2" t="s">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="K99" s="2" t="s">
         <v>455</v>
@@ -5288,7 +5288,7 @@
     </row>
     <row r="100">
       <c r="A100" s="2" t="s">
-        <v>510</v>
+        <v>511</v>
       </c>
       <c r="B100" s="2" t="s">
         <v>12</v>
@@ -5300,7 +5300,7 @@
         <v>58</v>
       </c>
       <c r="E100" s="2" t="s">
-        <v>511</v>
+        <v>71</v>
       </c>
       <c r="F100" s="2" t="s">
         <v>16</v>

</xml_diff>